<commit_message>
Establish GUI backend exchange contract
</commit_message>
<xml_diff>
--- a/docs/SCLAS_GUI_VARIABLE_REGISTER_20260708.xlsx
+++ b/docs/SCLAS_GUI_VARIABLE_REGISTER_20260708.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rbb204b459e5c459c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GUI Inputs" sheetId="2" r:id="Rf7c76b08048244f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="3" r:id="R9ba1bfe7b79c4018"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Internal Derived" sheetId="4" r:id="Ra165efd4d6404d3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend Payload" sheetId="5" r:id="R1dbaf5e306364c6d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Removed Hidden" sheetId="6" r:id="Ra704650b91ed41c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R2ef8efe9e4d049b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GUI Inputs" sheetId="2" r:id="Ra10e28dccea0497b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="3" r:id="R2087d3834ac94115"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Internal Derived" sheetId="4" r:id="R9029851a68824c6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backend Payload" sheetId="5" r:id="Rb0ef85151c894ce4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Removed Hidden" sheetId="6" r:id="Red4a9b53a9bd4aab"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -21,7 +21,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="0.00"/>
   </x:numFmts>
-  <x:fonts count="8">
+  <x:fonts count="11">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -64,8 +64,24 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Segoe UI"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF17202A"/>
+      <x:name val="Segoe UI"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF17202A"/>
+      <x:name val="Segoe UI"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF17202A"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -87,8 +103,13 @@
         <x:fgColor rgb="FF1D4ED8"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF334155"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="11">
+  <x:borders count="12">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -194,11 +215,25 @@
         <x:color rgb="FFE2E8F0"/>
       </x:top>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD8E0EA"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD8E0EA"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD8E0EA"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD8E0EA"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="52">
+  <x:cellXfs count="71">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -326,6 +361,69 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
       <x:extLst>
         <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -552,8 +650,8 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="120" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="93" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="114.37999725341797" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="16.799999237060547" hidden="0" customHeight="1">
@@ -566,13 +664,13 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="35" t="str">
-        <x:v>Reviewed 2026-07-08 KST. Source files: code/sclas_remote_gui.py, code/sclas_backend_gui_bridge.py, code/abaqus_runner.py.</x:v>
+        <x:v>Reviewed 2026-07-09 KST. Source files: code/sclas_remote_gui.py, code/sclas_backend_gui_bridge.py, code/abaqus_runner.py.</x:v>
       </x:c>
       <x:c r="B2" s="35" t="str">
-        <x:v>Reviewed 2026-07-08 KST. Source files: code/sclas_remote_gui.py, code/sclas_backend_gui_bridge.py, code/abaqus_runner.py.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3">
+        <x:v>Reviewed 2026-07-09 KST. Source files: code/sclas_remote_gui.py, code/sclas_backend_gui_bridge.py, code/abaqus_runner.py.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
       <x:c r="A3" s="36"/>
       <x:c r="B3" s="36"/>
     </x:row>
@@ -589,7 +687,7 @@
         <x:v>Reviewed at</x:v>
       </x:c>
       <x:c r="B5" s="39" t="str">
-        <x:v>2026-07-08 KST</x:v>
+        <x:v>2026-07-09 KST</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -658,10 +756,10 @@
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="42" t="str">
-        <x:v>Generated workbook</x:v>
+        <x:v>Exchange contract</x:v>
       </x:c>
       <x:c r="B14" s="43" t="str">
-        <x:v>SCLAS_GUI_VARIABLE_REGISTER_20260708.xlsx</x:v>
+        <x:v>Added core count, pitch length, auto effective length, global axial n_z, and backend_exchange_contract baseline.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -677,16 +775,16 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="38" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="48" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="24" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="68" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="41.380001068115234" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="41.380001068115234" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="41.380001068115234" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="41.380001068115234" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="41.380001068115234" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="41.380001068115234" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="41.380001068115234" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="73" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="41.380001068115234" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="60.880001068115234" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="16.799999237060547" hidden="0" customHeight="1">
@@ -753,7 +851,7 @@
         <x:v>Variables that a user can edit directly in the current GUI.</x:v>
       </x:c>
     </x:row>
-    <x:row r="3">
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
       <x:c r="A3" s="36"/>
       <x:c r="B3" s="36"/>
       <x:c r="C3" s="36"/>
@@ -766,996 +864,976 @@
       <x:c r="J3" s="36"/>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="37" t="str">
+      <x:c r="A4" s="62" t="str">
         <x:v>Tab</x:v>
       </x:c>
-      <x:c r="B4" s="37" t="str">
+      <x:c r="B4" s="62" t="str">
         <x:v>Section</x:v>
       </x:c>
-      <x:c r="C4" s="37" t="str">
+      <x:c r="C4" s="62" t="str">
         <x:v>GUI Label</x:v>
       </x:c>
-      <x:c r="D4" s="37" t="str">
+      <x:c r="D4" s="62" t="str">
         <x:v>Widget Key</x:v>
       </x:c>
-      <x:c r="E4" s="37" t="str">
+      <x:c r="E4" s="62" t="str">
         <x:v>Widget Type</x:v>
       </x:c>
-      <x:c r="F4" s="37" t="str">
+      <x:c r="F4" s="62" t="str">
         <x:v>Default</x:v>
       </x:c>
-      <x:c r="G4" s="37" t="str">
+      <x:c r="G4" s="62" t="str">
         <x:v>Unit</x:v>
       </x:c>
-      <x:c r="H4" s="37" t="str">
+      <x:c r="H4" s="62" t="str">
         <x:v>Payload Path</x:v>
       </x:c>
-      <x:c r="I4" s="37" t="str">
+      <x:c r="I4" s="62" t="str">
         <x:v>Source Type</x:v>
       </x:c>
-      <x:c r="J4" s="37" t="str">
+      <x:c r="J4" s="62" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
-      <x:c r="A5" s="38" t="str">
+      <x:c r="A5" s="60" t="str">
         <x:v>Design</x:v>
       </x:c>
-      <x:c r="B5" s="45" t="str">
+      <x:c r="B5" s="60" t="str">
         <x:v>Core Section</x:v>
       </x:c>
-      <x:c r="C5" s="45" t="str">
+      <x:c r="C5" s="60" t="str">
         <x:v>Conductor radius r_cond</x:v>
       </x:c>
-      <x:c r="D5" s="45" t="str">
+      <x:c r="D5" s="60" t="str">
         <x:v>r_cond</x:v>
       </x:c>
-      <x:c r="E5" s="45" t="str">
+      <x:c r="E5" s="60" t="str">
         <x:v>QLineEdit</x:v>
       </x:c>
-      <x:c r="F5" s="45" t="n">
+      <x:c r="F5" s="60" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="G5" s="45" t="str">
+      <x:c r="G5" s="60" t="str">
         <x:v>mm</x:v>
       </x:c>
-      <x:c r="H5" s="45" t="str">
+      <x:c r="H5" s="60" t="str">
         <x:v>geometry_mm.conductor_radius_mm</x:v>
       </x:c>
-      <x:c r="I5" s="45" t="str">
+      <x:c r="I5" s="60" t="str">
         <x:v>User editable</x:v>
       </x:c>
-      <x:c r="J5" s="39" t="str">
+      <x:c r="J5" s="60" t="str">
         <x:v>Conductor radius used in geometry and preview.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
-      <x:c r="A6" s="40" t="str">
+      <x:c r="A6" s="60" t="str">
         <x:v>Design</x:v>
       </x:c>
-      <x:c r="B6" s="46" t="str">
+      <x:c r="B6" s="60" t="str">
         <x:v>Core Section</x:v>
       </x:c>
-      <x:c r="C6" s="46" t="str">
+      <x:c r="C6" s="60" t="str">
         <x:v>Insulation radius r_ins</x:v>
       </x:c>
-      <x:c r="D6" s="46" t="str">
+      <x:c r="D6" s="60" t="str">
         <x:v>r_insu</x:v>
       </x:c>
-      <x:c r="E6" s="46" t="str">
+      <x:c r="E6" s="60" t="str">
         <x:v>QLineEdit</x:v>
       </x:c>
-      <x:c r="F6" s="46" t="n">
+      <x:c r="F6" s="60" t="n">
         <x:v>11.3</x:v>
       </x:c>
-      <x:c r="G6" s="46" t="str">
+      <x:c r="G6" s="60" t="str">
         <x:v>mm</x:v>
       </x:c>
-      <x:c r="H6" s="46" t="str">
+      <x:c r="H6" s="60" t="str">
         <x:v>geometry_mm.insulation_radius_mm</x:v>
       </x:c>
-      <x:c r="I6" s="46" t="str">
+      <x:c r="I6" s="60" t="str">
         <x:v>User editable</x:v>
       </x:c>
-      <x:c r="J6" s="41" t="str">
+      <x:c r="J6" s="60" t="str">
         <x:v>Insulation radius; must satisfy r_cond &lt; r_ins &lt;= R_core.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="40" t="str">
+      <x:c r="A7" s="60" t="str">
         <x:v>Design</x:v>
       </x:c>
-      <x:c r="B7" s="46" t="str">
+      <x:c r="B7" s="60" t="str">
         <x:v>Core Section</x:v>
       </x:c>
-      <x:c r="C7" s="46" t="str">
+      <x:c r="C7" s="60" t="str">
         <x:v>Core outer radius R_core</x:v>
       </x:c>
-      <x:c r="D7" s="46" t="str">
+      <x:c r="D7" s="60" t="str">
         <x:v>roc</x:v>
       </x:c>
-      <x:c r="E7" s="46" t="str">
+      <x:c r="E7" s="60" t="str">
         <x:v>QLineEdit</x:v>
       </x:c>
-      <x:c r="F7" s="46" t="n">
+      <x:c r="F7" s="60" t="n">
         <x:v>15.3</x:v>
       </x:c>
-      <x:c r="G7" s="46" t="str">
+      <x:c r="G7" s="60" t="str">
         <x:v>mm</x:v>
       </x:c>
-      <x:c r="H7" s="46" t="str">
+      <x:c r="H7" s="60" t="str">
         <x:v>geometry_mm.core_outer_radius_mm</x:v>
       </x:c>
-      <x:c r="I7" s="46" t="str">
+      <x:c r="I7" s="60" t="str">
         <x:v>User editable</x:v>
       </x:c>
-      <x:c r="J7" s="41" t="str">
-        <x:v>Core package outer radius. Core center radius is auto-derived.</x:v>
+      <x:c r="J7" s="60" t="str">
+        <x:v>Core section outer radius. Core center radius is auto-derived.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
-      <x:c r="A8" s="40" t="str">
+      <x:c r="A8" s="60" t="str">
         <x:v>Design</x:v>
       </x:c>
-      <x:c r="B8" s="46" t="str">
+      <x:c r="B8" s="60" t="str">
+        <x:v>Core Section</x:v>
+      </x:c>
+      <x:c r="C8" s="60" t="str">
+        <x:v>Core count n_core</x:v>
+      </x:c>
+      <x:c r="D8" s="60" t="str">
+        <x:v>core_count</x:v>
+      </x:c>
+      <x:c r="E8" s="60" t="str">
+        <x:v>QSpinBox</x:v>
+      </x:c>
+      <x:c r="F8" s="60" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G8" s="60" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="H8" s="60" t="str">
+        <x:v>geometry_mm.core_count</x:v>
+      </x:c>
+      <x:c r="I8" s="60" t="str">
+        <x:v>User editable</x:v>
+      </x:c>
+      <x:c r="J8" s="60" t="str">
+        <x:v>Default 3; passed to backend job setup and used for auto effective length.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="60" t="str">
+        <x:v>Design</x:v>
+      </x:c>
+      <x:c r="B9" s="60" t="str">
         <x:v>Sheath / Bedding</x:v>
       </x:c>
-      <x:c r="C8" s="46" t="str">
+      <x:c r="C9" s="60" t="str">
         <x:v>Inner sheath t_is</x:v>
       </x:c>
-      <x:c r="D8" s="46" t="str">
+      <x:c r="D9" s="60" t="str">
         <x:v>tis</x:v>
       </x:c>
-      <x:c r="E8" s="46" t="str">
+      <x:c r="E9" s="60" t="str">
         <x:v>QLineEdit</x:v>
       </x:c>
-      <x:c r="F8" s="46" t="n">
+      <x:c r="F9" s="60" t="n">
         <x:v>4.5</x:v>
       </x:c>
-      <x:c r="G8" s="46" t="str">
+      <x:c r="G9" s="60" t="str">
         <x:v>mm</x:v>
       </x:c>
-      <x:c r="H8" s="46" t="str">
+      <x:c r="H9" s="60" t="str">
         <x:v>geometry_mm.inner_sheath_thickness_mm</x:v>
       </x:c>
-      <x:c r="I8" s="46" t="str">
+      <x:c r="I9" s="60" t="str">
         <x:v>User editable</x:v>
       </x:c>
-      <x:c r="J8" s="41" t="str">
+      <x:c r="J9" s="60" t="str">
         <x:v>Inner sheath thickness.</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="15" hidden="0" customHeight="1">
-      <x:c r="A9" s="40" t="str">
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="60" t="str">
         <x:v>Design</x:v>
       </x:c>
-      <x:c r="B9" s="46" t="str">
+      <x:c r="B10" s="60" t="str">
         <x:v>Sheath / Bedding</x:v>
       </x:c>
-      <x:c r="C9" s="46" t="str">
+      <x:c r="C10" s="60" t="str">
         <x:v>Bedding thickness t_bedding</x:v>
       </x:c>
-      <x:c r="D9" s="46" t="str">
+      <x:c r="D10" s="60" t="str">
         <x:v>bedding_thickness</x:v>
       </x:c>
-      <x:c r="E9" s="46" t="str">
+      <x:c r="E10" s="60" t="str">
         <x:v>QLineEdit</x:v>
       </x:c>
-      <x:c r="F9" s="46" t="n">
+      <x:c r="F10" s="60" t="n">
         <x:v>0.6</x:v>
       </x:c>
-      <x:c r="G9" s="46" t="str">
+      <x:c r="G10" s="60" t="str">
         <x:v>mm</x:v>
       </x:c>
-      <x:c r="H9" s="46" t="str">
+      <x:c r="H10" s="60" t="str">
         <x:v>geometry_mm.bedding_thickness_mm</x:v>
       </x:c>
-      <x:c r="I9" s="46" t="str">
+      <x:c r="I10" s="60" t="str">
         <x:v>User editable</x:v>
       </x:c>
-      <x:c r="J9" s="41" t="str">
+      <x:c r="J10" s="60" t="str">
         <x:v>Bedding thickness between armour layers.</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="15" hidden="0" customHeight="1">
-      <x:c r="A10" s="40" t="str">
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="A11" s="60" t="str">
         <x:v>Design</x:v>
       </x:c>
-      <x:c r="B10" s="46" t="str">
+      <x:c r="B11" s="60" t="str">
         <x:v>Sheath / Bedding</x:v>
       </x:c>
-      <x:c r="C10" s="46" t="str">
+      <x:c r="C11" s="60" t="str">
         <x:v>Outer sheath t_os</x:v>
       </x:c>
-      <x:c r="D10" s="46" t="str">
+      <x:c r="D11" s="60" t="str">
         <x:v>tos</x:v>
       </x:c>
-      <x:c r="E10" s="46" t="str">
+      <x:c r="E11" s="60" t="str">
         <x:v>QLineEdit</x:v>
       </x:c>
-      <x:c r="F10" s="46" t="n">
+      <x:c r="F11" s="60" t="n">
         <x:v>4.5</x:v>
       </x:c>
-      <x:c r="G10" s="46" t="str">
+      <x:c r="G11" s="60" t="str">
         <x:v>mm</x:v>
       </x:c>
-      <x:c r="H10" s="46" t="str">
+      <x:c r="H11" s="60" t="str">
         <x:v>geometry_mm.outer_sheath_thickness_mm</x:v>
       </x:c>
-      <x:c r="I10" s="46" t="str">
+      <x:c r="I11" s="60" t="str">
         <x:v>User editable</x:v>
       </x:c>
-      <x:c r="J10" s="41" t="str">
+      <x:c r="J11" s="60" t="str">
         <x:v>Outer sheath thickness.</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="15" hidden="0" customHeight="1">
-      <x:c r="A11" s="40" t="str">
+    <x:row r="12" ht="15" hidden="0" customHeight="1">
+      <x:c r="A12" s="60" t="str">
         <x:v>Design</x:v>
       </x:c>
-      <x:c r="B11" s="46" t="str">
+      <x:c r="B12" s="60" t="str">
         <x:v>Armour</x:v>
       </x:c>
-      <x:c r="C11" s="46" t="str">
+      <x:c r="C12" s="60" t="str">
         <x:v>Inner armour radius r_ia</x:v>
       </x:c>
-      <x:c r="D11" s="46" t="str">
+      <x:c r="D12" s="60" t="str">
         <x:v>r_ia</x:v>
       </x:c>
-      <x:c r="E11" s="46" t="str">
+      <x:c r="E12" s="60" t="str">
         <x:v>QLineEdit</x:v>
       </x:c>
-      <x:c r="F11" s="46" t="n">
+      <x:c r="F12" s="60" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="G11" s="46" t="str">
+      <x:c r="G12" s="60" t="str">
         <x:v>mm</x:v>
       </x:c>
-      <x:c r="H11" s="46" t="str">
+      <x:c r="H12" s="60" t="str">
         <x:v>armour.inner_wire_radius_mm</x:v>
       </x:c>
-      <x:c r="I11" s="46" t="str">
+      <x:c r="I12" s="60" t="str">
         <x:v>User editable</x:v>
       </x:c>
-      <x:c r="J11" s="41" t="str">
+      <x:c r="J12" s="60" t="str">
         <x:v>Inner armour radius.</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="15" hidden="0" customHeight="1">
-      <x:c r="A12" s="40" t="str">
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
+      <x:c r="A13" s="60" t="str">
         <x:v>Design</x:v>
       </x:c>
-      <x:c r="B12" s="46" t="str">
+      <x:c r="B13" s="60" t="str">
         <x:v>Armour</x:v>
       </x:c>
-      <x:c r="C12" s="46" t="str">
+      <x:c r="C13" s="60" t="str">
         <x:v>Inner armour number n_ia</x:v>
       </x:c>
-      <x:c r="D12" s="46" t="str">
+      <x:c r="D13" s="60" t="str">
         <x:v>no_ia</x:v>
       </x:c>
-      <x:c r="E12" s="46" t="str">
+      <x:c r="E13" s="60" t="str">
         <x:v>QSpinBox</x:v>
       </x:c>
-      <x:c r="F12" s="46" t="n">
+      <x:c r="F13" s="60" t="n">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="G12" s="46" t="str">
+      <x:c r="G13" s="60" t="str">
         <x:v>count</x:v>
       </x:c>
-      <x:c r="H12" s="46" t="str">
+      <x:c r="H13" s="60" t="str">
         <x:v>armour.inner_wire_count</x:v>
       </x:c>
-      <x:c r="I12" s="46" t="str">
+      <x:c r="I13" s="60" t="str">
         <x:v>User editable with clamp</x:v>
       </x:c>
-      <x:c r="J12" s="41" t="str">
+      <x:c r="J13" s="60" t="str">
         <x:v>Default 55; clamped by n &lt;= pi/asin(r_wire/R_center). 0 means Auto.</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="15" hidden="0" customHeight="1">
-      <x:c r="A13" s="40" t="str">
+    <x:row r="14" ht="15" hidden="0" customHeight="1">
+      <x:c r="A14" s="60" t="str">
         <x:v>Design</x:v>
       </x:c>
-      <x:c r="B13" s="46" t="str">
+      <x:c r="B14" s="60" t="str">
         <x:v>Armour</x:v>
       </x:c>
-      <x:c r="C13" s="46" t="str">
+      <x:c r="C14" s="60" t="str">
         <x:v>Outer armour radius r_oa</x:v>
       </x:c>
-      <x:c r="D13" s="46" t="str">
+      <x:c r="D14" s="60" t="str">
         <x:v>r_oa</x:v>
       </x:c>
-      <x:c r="E13" s="46" t="str">
+      <x:c r="E14" s="60" t="str">
         <x:v>QLineEdit</x:v>
       </x:c>
-      <x:c r="F13" s="46" t="n">
+      <x:c r="F14" s="60" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="G13" s="46" t="str">
+      <x:c r="G14" s="60" t="str">
         <x:v>mm</x:v>
       </x:c>
-      <x:c r="H13" s="46" t="str">
+      <x:c r="H14" s="60" t="str">
         <x:v>armour.outer_wire_radius_mm</x:v>
       </x:c>
-      <x:c r="I13" s="46" t="str">
+      <x:c r="I14" s="60" t="str">
         <x:v>User editable</x:v>
       </x:c>
-      <x:c r="J13" s="41" t="str">
+      <x:c r="J14" s="60" t="str">
         <x:v>Outer armour radius.</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="15" hidden="0" customHeight="1">
-      <x:c r="A14" s="40" t="str">
+    <x:row r="15" ht="15" hidden="0" customHeight="1">
+      <x:c r="A15" s="60" t="str">
         <x:v>Design</x:v>
       </x:c>
-      <x:c r="B14" s="46" t="str">
+      <x:c r="B15" s="60" t="str">
         <x:v>Armour</x:v>
       </x:c>
-      <x:c r="C14" s="46" t="str">
+      <x:c r="C15" s="60" t="str">
         <x:v>Outer armour number n_oa</x:v>
       </x:c>
-      <x:c r="D14" s="46" t="str">
+      <x:c r="D15" s="60" t="str">
         <x:v>no_oa</x:v>
       </x:c>
-      <x:c r="E14" s="46" t="str">
+      <x:c r="E15" s="60" t="str">
         <x:v>QSpinBox</x:v>
       </x:c>
-      <x:c r="F14" s="46" t="n">
+      <x:c r="F15" s="60" t="n">
         <x:v>63</x:v>
       </x:c>
-      <x:c r="G14" s="46" t="str">
+      <x:c r="G15" s="60" t="str">
         <x:v>count</x:v>
       </x:c>
-      <x:c r="H14" s="46" t="str">
+      <x:c r="H15" s="60" t="str">
         <x:v>armour.outer_wire_count</x:v>
       </x:c>
-      <x:c r="I14" s="46" t="str">
+      <x:c r="I15" s="60" t="str">
         <x:v>User editable with clamp</x:v>
       </x:c>
-      <x:c r="J14" s="41" t="str">
+      <x:c r="J15" s="60" t="str">
         <x:v>Default 63; clamped by n &lt;= pi/asin(r_wire/R_center). 0 means Auto.</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="15" hidden="0" customHeight="1">
-      <x:c r="A15" s="40" t="str">
+    <x:row r="16" ht="15" hidden="0" customHeight="1">
+      <x:c r="A16" s="60" t="str">
         <x:v>Design</x:v>
       </x:c>
-      <x:c r="B15" s="46" t="str">
+      <x:c r="B16" s="60" t="str">
         <x:v>Helix Pitch Angle</x:v>
       </x:c>
-      <x:c r="C15" s="46" t="str">
-        <x:v>Core helix pitch angle α_core</x:v>
-      </x:c>
-      <x:c r="D15" s="46" t="str">
+      <x:c r="C16" s="60" t="str">
+        <x:v>Core helix pitch angle alpha_core</x:v>
+      </x:c>
+      <x:c r="D16" s="60" t="str">
         <x:v>core_lay_angle</x:v>
       </x:c>
-      <x:c r="E15" s="46" t="str">
+      <x:c r="E16" s="60" t="str">
         <x:v>QLineEdit</x:v>
       </x:c>
-      <x:c r="F15" s="46" t="n">
+      <x:c r="F16" s="60" t="n">
         <x:v>8.98</x:v>
       </x:c>
-      <x:c r="G15" s="46" t="str">
+      <x:c r="G16" s="60" t="str">
         <x:v>deg</x:v>
       </x:c>
-      <x:c r="H15" s="46" t="str">
+      <x:c r="H16" s="60" t="str">
         <x:v>armour.core_lay_angle_deg</x:v>
       </x:c>
-      <x:c r="I15" s="46" t="str">
+      <x:c r="I16" s="60" t="str">
         <x:v>User editable</x:v>
       </x:c>
-      <x:c r="J15" s="41" t="str">
-        <x:v>Core helix pitch angle.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="15" hidden="0" customHeight="1">
-      <x:c r="A16" s="40" t="str">
+      <x:c r="J16" s="60" t="str">
+        <x:v>GUI computes core pitch length from this angle and core center radius.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="15" hidden="0" customHeight="1">
+      <x:c r="A17" s="60" t="str">
         <x:v>Design</x:v>
       </x:c>
-      <x:c r="B16" s="46" t="str">
+      <x:c r="B17" s="60" t="str">
         <x:v>Helix Pitch Angle</x:v>
       </x:c>
-      <x:c r="C16" s="46" t="str">
-        <x:v>Inner armour helix pitch angle α_ia</x:v>
-      </x:c>
-      <x:c r="D16" s="46" t="str">
+      <x:c r="C17" s="60" t="str">
+        <x:v>Inner armour helix pitch angle alpha_ia</x:v>
+      </x:c>
+      <x:c r="D17" s="60" t="str">
         <x:v>inner_lay_angle</x:v>
       </x:c>
-      <x:c r="E16" s="46" t="str">
+      <x:c r="E17" s="60" t="str">
         <x:v>QLineEdit</x:v>
       </x:c>
-      <x:c r="F16" s="46" t="n">
+      <x:c r="F17" s="60" t="n">
         <x:v>20.1</x:v>
       </x:c>
-      <x:c r="G16" s="46" t="str">
+      <x:c r="G17" s="60" t="str">
         <x:v>deg</x:v>
       </x:c>
-      <x:c r="H16" s="46" t="str">
+      <x:c r="H17" s="60" t="str">
         <x:v>armour.inner_lay_angle_deg / inner_armour_lay_angle_deg</x:v>
       </x:c>
-      <x:c r="I16" s="46" t="str">
+      <x:c r="I17" s="60" t="str">
         <x:v>User editable</x:v>
       </x:c>
-      <x:c r="J16" s="41" t="str">
-        <x:v>Inner armour helix pitch angle.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="15" hidden="0" customHeight="1">
-      <x:c r="A17" s="40" t="str">
+      <x:c r="J17" s="60" t="str">
+        <x:v>GUI computes inner armour pitch length from this angle and center radius.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
+      <x:c r="A18" s="60" t="str">
         <x:v>Design</x:v>
       </x:c>
-      <x:c r="B17" s="46" t="str">
+      <x:c r="B18" s="60" t="str">
         <x:v>Helix Pitch Angle</x:v>
       </x:c>
-      <x:c r="C17" s="46" t="str">
-        <x:v>Outer armour helix pitch angle α_oa</x:v>
-      </x:c>
-      <x:c r="D17" s="46" t="str">
+      <x:c r="C18" s="60" t="str">
+        <x:v>Outer armour helix pitch angle alpha_oa</x:v>
+      </x:c>
+      <x:c r="D18" s="60" t="str">
         <x:v>outer_lay_angle</x:v>
       </x:c>
-      <x:c r="E17" s="46" t="str">
+      <x:c r="E18" s="60" t="str">
         <x:v>QLineEdit</x:v>
       </x:c>
-      <x:c r="F17" s="46" t="n">
+      <x:c r="F18" s="60" t="n">
         <x:v>19.6</x:v>
       </x:c>
-      <x:c r="G17" s="46" t="str">
+      <x:c r="G18" s="60" t="str">
         <x:v>deg</x:v>
       </x:c>
-      <x:c r="H17" s="46" t="str">
+      <x:c r="H18" s="60" t="str">
         <x:v>armour.outer_lay_angle_deg / outer_armour_lay_angle_deg</x:v>
       </x:c>
-      <x:c r="I17" s="46" t="str">
+      <x:c r="I18" s="60" t="str">
         <x:v>User editable</x:v>
       </x:c>
-      <x:c r="J17" s="41" t="str">
-        <x:v>Outer armour helix pitch angle.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="15" hidden="0" customHeight="1">
-      <x:c r="A18" s="40" t="str">
+      <x:c r="J18" s="60" t="str">
+        <x:v>GUI computes outer armour pitch length from this angle and center radius.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="15" hidden="0" customHeight="1">
+      <x:c r="A19" s="60" t="str">
         <x:v>Finite Element Analysis Setting</x:v>
       </x:c>
-      <x:c r="B18" s="46" t="str">
+      <x:c r="B19" s="60" t="str">
         <x:v>Analysis Structure Setup</x:v>
       </x:c>
-      <x:c r="C18" s="46" t="str">
+      <x:c r="C19" s="60" t="str">
         <x:v>External pressure load</x:v>
       </x:c>
-      <x:c r="D18" s="46" t="str">
+      <x:c r="D19" s="60" t="str">
         <x:v>pressure</x:v>
       </x:c>
-      <x:c r="E18" s="46" t="str">
+      <x:c r="E19" s="60" t="str">
         <x:v>QLineEdit</x:v>
       </x:c>
-      <x:c r="F18" s="46" t="n">
+      <x:c r="F19" s="60" t="n">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="G18" s="46" t="str">
+      <x:c r="G19" s="60" t="str">
         <x:v>MPa</x:v>
       </x:c>
-      <x:c r="H18" s="46" t="str">
+      <x:c r="H19" s="60" t="str">
         <x:v>analysis_conditions.external_pressure_mpa / hydrostatic_pressure_mpa</x:v>
       </x:c>
-      <x:c r="I18" s="46" t="str">
+      <x:c r="I19" s="60" t="str">
         <x:v>User editable</x:v>
       </x:c>
-      <x:c r="J18" s="41" t="str">
+      <x:c r="J19" s="60" t="str">
         <x:v>Primary pressure/load input; visible on tab 2.</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="15" hidden="0" customHeight="1">
-      <x:c r="A19" s="40" t="str">
+    <x:row r="20" ht="15" hidden="0" customHeight="1">
+      <x:c r="A20" s="60" t="str">
         <x:v>Finite Element Analysis Setting</x:v>
       </x:c>
-      <x:c r="B19" s="46" t="str">
+      <x:c r="B20" s="60" t="str">
         <x:v>Analysis Structure Setup</x:v>
       </x:c>
-      <x:c r="C19" s="46" t="str">
-        <x:v>Target curvature κ</x:v>
-      </x:c>
-      <x:c r="D19" s="46" t="str">
+      <x:c r="C20" s="60" t="str">
+        <x:v>Target curvature kappa</x:v>
+      </x:c>
+      <x:c r="D20" s="60" t="str">
         <x:v>curvature</x:v>
       </x:c>
-      <x:c r="E19" s="46" t="str">
+      <x:c r="E20" s="60" t="str">
         <x:v>QLineEdit</x:v>
       </x:c>
-      <x:c r="F19" s="46" t="n">
+      <x:c r="F20" s="60" t="n">
         <x:v>0.08</x:v>
       </x:c>
-      <x:c r="G19" s="46" t="str">
+      <x:c r="G20" s="60" t="str">
         <x:v>1/m</x:v>
       </x:c>
-      <x:c r="H19" s="46" t="str">
+      <x:c r="H20" s="60" t="str">
         <x:v>analysis_conditions.max_curvature_1_per_m</x:v>
       </x:c>
-      <x:c r="I19" s="46" t="str">
+      <x:c r="I20" s="60" t="str">
         <x:v>User editable</x:v>
       </x:c>
-      <x:c r="J19" s="41" t="str">
+      <x:c r="J20" s="60" t="str">
         <x:v>Target bending curvature; visible on tab 2.</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="15" hidden="0" customHeight="1">
-      <x:c r="A20" s="40" t="str">
+    <x:row r="21" ht="15" hidden="0" customHeight="1">
+      <x:c r="A21" s="60" t="str">
         <x:v>Finite Element Analysis Setting</x:v>
       </x:c>
-      <x:c r="B20" s="46" t="str">
+      <x:c r="B21" s="60" t="str">
         <x:v>Analysis Structure Setup</x:v>
       </x:c>
-      <x:c r="C20" s="46" t="str">
-        <x:v>Friction coefficient μ</x:v>
-      </x:c>
-      <x:c r="D20" s="46" t="str">
+      <x:c r="C21" s="60" t="str">
+        <x:v>Friction coefficient mu</x:v>
+      </x:c>
+      <x:c r="D21" s="60" t="str">
         <x:v>friction</x:v>
       </x:c>
-      <x:c r="E20" s="46" t="str">
+      <x:c r="E21" s="60" t="str">
         <x:v>QLineEdit</x:v>
       </x:c>
-      <x:c r="F20" s="46" t="n">
+      <x:c r="F21" s="60" t="n">
         <x:v>0.22</x:v>
       </x:c>
-      <x:c r="G20" s="46" t="str">
+      <x:c r="G21" s="60" t="str">
         <x:v>-</x:v>
       </x:c>
-      <x:c r="H20" s="46" t="str">
+      <x:c r="H21" s="60" t="str">
         <x:v>analysis_conditions.friction_coefficient</x:v>
       </x:c>
-      <x:c r="I20" s="46" t="str">
+      <x:c r="I21" s="60" t="str">
         <x:v>User editable</x:v>
       </x:c>
-      <x:c r="J20" s="41" t="str">
+      <x:c r="J21" s="60" t="str">
         <x:v>Coulomb friction coefficient; visible on tab 2.</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="15" hidden="0" customHeight="1">
-      <x:c r="A21" s="40" t="str">
+    <x:row r="22" ht="15" hidden="0" customHeight="1">
+      <x:c r="A22" s="60" t="str">
         <x:v>Finite Element Analysis Setting</x:v>
       </x:c>
-      <x:c r="B21" s="46" t="str">
+      <x:c r="B22" s="60" t="str">
         <x:v>Mesh Setting Guide</x:v>
       </x:c>
-      <x:c r="C21" s="46" t="str">
+      <x:c r="C22" s="60" t="str">
         <x:v>Abaqus element type</x:v>
       </x:c>
-      <x:c r="D21" s="46" t="str">
+      <x:c r="D22" s="60" t="str">
         <x:v>elem_type</x:v>
       </x:c>
-      <x:c r="E21" s="46" t="str">
+      <x:c r="E22" s="60" t="str">
         <x:v>QComboBox</x:v>
       </x:c>
-      <x:c r="F21" s="46" t="str">
+      <x:c r="F22" s="60" t="str">
         <x:v>C3D8R</x:v>
       </x:c>
-      <x:c r="G21" s="46" t="str">
+      <x:c r="G22" s="60" t="str">
         <x:v>-</x:v>
       </x:c>
-      <x:c r="H21" s="46" t="str">
+      <x:c r="H22" s="60" t="str">
         <x:v>mesh.requested_element_type / solid_element_type</x:v>
       </x:c>
-      <x:c r="I21" s="46" t="str">
+      <x:c r="I22" s="60" t="str">
         <x:v>User editable</x:v>
       </x:c>
-      <x:c r="J21" s="41" t="str">
+      <x:c r="J22" s="60" t="str">
         <x:v>Requested Abaqus element type. GUI options currently include C3D8R, C3D4, B31.</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="15" hidden="0" customHeight="1">
-      <x:c r="A22" s="40" t="str">
+    <x:row r="23" ht="15" hidden="0" customHeight="1">
+      <x:c r="A23" s="60" t="str">
         <x:v>Finite Element Analysis Setting</x:v>
       </x:c>
-      <x:c r="B22" s="46" t="str">
+      <x:c r="B23" s="60" t="str">
         <x:v>Mesh Setting Guide</x:v>
       </x:c>
-      <x:c r="C22" s="46" t="str">
-        <x:v>Axial n_z divisions</x:v>
-      </x:c>
-      <x:c r="D22" s="46" t="str">
+      <x:c r="C23" s="60" t="str">
+        <x:v>Global axial n_z divisions</x:v>
+      </x:c>
+      <x:c r="D23" s="60" t="str">
         <x:v>z_elem</x:v>
       </x:c>
-      <x:c r="E22" s="46" t="str">
+      <x:c r="E23" s="60" t="str">
         <x:v>QSpinBox</x:v>
       </x:c>
-      <x:c r="F22" s="46" t="n">
+      <x:c r="F23" s="60" t="n">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="G22" s="46" t="str">
+      <x:c r="G23" s="60" t="str">
         <x:v>count</x:v>
       </x:c>
-      <x:c r="H22" s="46" t="str">
+      <x:c r="H23" s="60" t="str">
         <x:v>mesh.axial_divisions; mesh_controls.*.z.count</x:v>
       </x:c>
-      <x:c r="I22" s="46" t="str">
+      <x:c r="I23" s="60" t="str">
         <x:v>User editable</x:v>
       </x:c>
-      <x:c r="J22" s="41" t="str">
-        <x:v>Axial divisions for core, sheath, bedding, and armour.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="15" hidden="0" customHeight="1">
-      <x:c r="A23" s="40" t="str">
+      <x:c r="J23" s="60" t="str">
+        <x:v>Single z-direction division count for core, sheath, bedding, armour, and filler.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="15" hidden="0" customHeight="1">
+      <x:c r="A24" s="60" t="str">
         <x:v>Finite Element Analysis Setting</x:v>
       </x:c>
-      <x:c r="B23" s="46" t="str">
+      <x:c r="B24" s="60" t="str">
         <x:v>Mesh Setting Guide</x:v>
       </x:c>
-      <x:c r="C23" s="46" t="str">
-        <x:v>Core/Sheath n_θ divisions</x:v>
-      </x:c>
-      <x:c r="D23" s="46" t="str">
+      <x:c r="C24" s="60" t="str">
+        <x:v>Core/Sheath n_theta divisions</x:v>
+      </x:c>
+      <x:c r="D24" s="60" t="str">
         <x:v>c_elem_core</x:v>
       </x:c>
-      <x:c r="E23" s="46" t="str">
+      <x:c r="E24" s="60" t="str">
         <x:v>QSpinBox</x:v>
       </x:c>
-      <x:c r="F23" s="46" t="n">
+      <x:c r="F24" s="60" t="n">
         <x:v>24</x:v>
       </x:c>
-      <x:c r="G23" s="46" t="str">
+      <x:c r="G24" s="60" t="str">
         <x:v>count</x:v>
       </x:c>
-      <x:c r="H23" s="46" t="str">
+      <x:c r="H24" s="60" t="str">
         <x:v>mesh.core_circumferential_divisions; mesh_controls.Core/Sheath/Bedding/OuterSheath.theta.count</x:v>
       </x:c>
-      <x:c r="I23" s="46" t="str">
+      <x:c r="I24" s="60" t="str">
         <x:v>User editable</x:v>
       </x:c>
-      <x:c r="J23" s="41" t="str">
+      <x:c r="J24" s="60" t="str">
         <x:v>Circumferential divisions for core/sheath/bedding.</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="15" hidden="0" customHeight="1">
-      <x:c r="A24" s="40" t="str">
+    <x:row r="25" ht="15" hidden="0" customHeight="1">
+      <x:c r="A25" s="60" t="str">
         <x:v>Finite Element Analysis Setting</x:v>
       </x:c>
-      <x:c r="B24" s="46" t="str">
+      <x:c r="B25" s="60" t="str">
         <x:v>Mesh Setting Guide</x:v>
       </x:c>
-      <x:c r="C24" s="46" t="str">
-        <x:v>Armour n_θ divisions</x:v>
-      </x:c>
-      <x:c r="D24" s="46" t="str">
+      <x:c r="C25" s="60" t="str">
+        <x:v>Armour n_theta divisions</x:v>
+      </x:c>
+      <x:c r="D25" s="60" t="str">
         <x:v>c_elem_armour</x:v>
       </x:c>
-      <x:c r="E24" s="46" t="str">
+      <x:c r="E25" s="60" t="str">
         <x:v>QSpinBox</x:v>
       </x:c>
-      <x:c r="F24" s="46" t="n">
+      <x:c r="F25" s="60" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="G24" s="46" t="str">
+      <x:c r="G25" s="60" t="str">
         <x:v>count</x:v>
       </x:c>
-      <x:c r="H24" s="46" t="str">
+      <x:c r="H25" s="60" t="str">
         <x:v>mesh.armour_circumferential_divisions; mesh_controls.InnerArmour/OuterArmour.theta.count</x:v>
       </x:c>
-      <x:c r="I24" s="46" t="str">
+      <x:c r="I25" s="60" t="str">
         <x:v>User editable</x:v>
       </x:c>
-      <x:c r="J24" s="41" t="str">
+      <x:c r="J25" s="60" t="str">
         <x:v>Circumferential divisions around armour cross-section.</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" ht="15" hidden="0" customHeight="1">
-      <x:c r="A25" s="40" t="str">
+    <x:row r="26" ht="15" hidden="0" customHeight="1">
+      <x:c r="A26" s="60" t="str">
         <x:v>Finite Element Analysis Setting</x:v>
       </x:c>
-      <x:c r="B25" s="46" t="str">
+      <x:c r="B26" s="60" t="str">
         <x:v>Mesh Setting Guide</x:v>
       </x:c>
-      <x:c r="C25" s="46" t="str">
+      <x:c r="C26" s="60" t="str">
         <x:v>Inner sheath n_r divisions</x:v>
       </x:c>
-      <x:c r="D25" s="46" t="str">
+      <x:c r="D26" s="60" t="str">
         <x:v>r_elem_inner_sheath</x:v>
       </x:c>
-      <x:c r="E25" s="46" t="str">
+      <x:c r="E26" s="60" t="str">
         <x:v>QSpinBox</x:v>
       </x:c>
-      <x:c r="F25" s="46" t="n">
+      <x:c r="F26" s="60" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="G25" s="46" t="str">
+      <x:c r="G26" s="60" t="str">
         <x:v>count</x:v>
       </x:c>
-      <x:c r="H25" s="46" t="str">
+      <x:c r="H26" s="60" t="str">
         <x:v>mesh.inner_sheath_radial_divisions</x:v>
       </x:c>
-      <x:c r="I25" s="46" t="str">
+      <x:c r="I26" s="60" t="str">
         <x:v>User editable</x:v>
       </x:c>
-      <x:c r="J25" s="41" t="str">
+      <x:c r="J26" s="60" t="str">
         <x:v>Radial divisions through inner sheath thickness.</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="15" hidden="0" customHeight="1">
-      <x:c r="A26" s="40" t="str">
+    <x:row r="27" ht="15" hidden="0" customHeight="1">
+      <x:c r="A27" s="60" t="str">
         <x:v>Finite Element Analysis Setting</x:v>
       </x:c>
-      <x:c r="B26" s="46" t="str">
+      <x:c r="B27" s="60" t="str">
         <x:v>Mesh Setting Guide</x:v>
       </x:c>
-      <x:c r="C26" s="46" t="str">
+      <x:c r="C27" s="60" t="str">
         <x:v>Bedding n_r divisions</x:v>
       </x:c>
-      <x:c r="D26" s="46" t="str">
+      <x:c r="D27" s="60" t="str">
         <x:v>r_elem_bedding</x:v>
       </x:c>
-      <x:c r="E26" s="46" t="str">
+      <x:c r="E27" s="60" t="str">
         <x:v>QSpinBox</x:v>
       </x:c>
-      <x:c r="F26" s="46" t="n">
+      <x:c r="F27" s="60" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="G26" s="46" t="str">
+      <x:c r="G27" s="60" t="str">
         <x:v>count</x:v>
       </x:c>
-      <x:c r="H26" s="46" t="str">
+      <x:c r="H27" s="60" t="str">
         <x:v>mesh.bedding_radial_divisions; mesh.radial_divisions_per_layer</x:v>
       </x:c>
-      <x:c r="I26" s="46" t="str">
+      <x:c r="I27" s="60" t="str">
         <x:v>User editable</x:v>
       </x:c>
-      <x:c r="J26" s="41" t="str">
+      <x:c r="J27" s="60" t="str">
         <x:v>Radial divisions through bedding layer.</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="15" hidden="0" customHeight="1">
-      <x:c r="A27" s="40" t="str">
+    <x:row r="28" ht="15" hidden="0" customHeight="1">
+      <x:c r="A28" s="60" t="str">
         <x:v>Finite Element Analysis Setting</x:v>
       </x:c>
-      <x:c r="B27" s="46" t="str">
+      <x:c r="B28" s="60" t="str">
         <x:v>Mesh Setting Guide</x:v>
       </x:c>
-      <x:c r="C27" s="46" t="str">
+      <x:c r="C28" s="60" t="str">
         <x:v>Outer sheath n_r divisions</x:v>
       </x:c>
-      <x:c r="D27" s="46" t="str">
+      <x:c r="D28" s="60" t="str">
         <x:v>r_elem_outer_sheath</x:v>
       </x:c>
-      <x:c r="E27" s="46" t="str">
+      <x:c r="E28" s="60" t="str">
         <x:v>QSpinBox</x:v>
       </x:c>
-      <x:c r="F27" s="46" t="n">
+      <x:c r="F28" s="60" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="G27" s="46" t="str">
+      <x:c r="G28" s="60" t="str">
         <x:v>count</x:v>
       </x:c>
-      <x:c r="H27" s="46" t="str">
+      <x:c r="H28" s="60" t="str">
         <x:v>mesh.outer_sheath_radial_divisions</x:v>
       </x:c>
-      <x:c r="I27" s="46" t="str">
+      <x:c r="I28" s="60" t="str">
         <x:v>User editable</x:v>
       </x:c>
-      <x:c r="J27" s="41" t="str">
+      <x:c r="J28" s="60" t="str">
         <x:v>Radial divisions through outer sheath thickness.</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" ht="15" hidden="0" customHeight="1">
-      <x:c r="A28" s="40" t="str">
-        <x:v>Finite Element Analysis Setting</x:v>
-      </x:c>
-      <x:c r="B28" s="46" t="str">
-        <x:v>Mesh Setting Guide</x:v>
-      </x:c>
-      <x:c r="C28" s="46" t="str">
-        <x:v>Filler n_z divisions</x:v>
-      </x:c>
-      <x:c r="D28" s="46" t="str">
-        <x:v>filler_z_elem</x:v>
-      </x:c>
-      <x:c r="E28" s="46" t="str">
+    <x:row r="29" ht="15" hidden="0" customHeight="1">
+      <x:c r="A29" s="60" t="str">
+        <x:v>Analysis</x:v>
+      </x:c>
+      <x:c r="B29" s="60" t="str">
+        <x:v>Conditions</x:v>
+      </x:c>
+      <x:c r="C29" s="60" t="str">
+        <x:v>Max twist</x:v>
+      </x:c>
+      <x:c r="D29" s="60" t="str">
+        <x:v>twist</x:v>
+      </x:c>
+      <x:c r="E29" s="60" t="str">
+        <x:v>QLineEdit</x:v>
+      </x:c>
+      <x:c r="F29" s="60" t="n">
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="G29" s="60" t="str">
+        <x:v>rad/m</x:v>
+      </x:c>
+      <x:c r="H29" s="60" t="str">
+        <x:v>analysis_conditions.max_twist_rad_per_m</x:v>
+      </x:c>
+      <x:c r="I29" s="60" t="str">
+        <x:v>User editable</x:v>
+      </x:c>
+      <x:c r="J29" s="60" t="str">
+        <x:v>Future coupled torsion request.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="15" hidden="0" customHeight="1">
+      <x:c r="A30" s="60" t="str">
+        <x:v>Analysis</x:v>
+      </x:c>
+      <x:c r="B30" s="60" t="str">
+        <x:v>Conditions</x:v>
+      </x:c>
+      <x:c r="C30" s="60" t="str">
+        <x:v>Max axial strain</x:v>
+      </x:c>
+      <x:c r="D30" s="60" t="str">
+        <x:v>axial_strain</x:v>
+      </x:c>
+      <x:c r="E30" s="60" t="str">
+        <x:v>QLineEdit</x:v>
+      </x:c>
+      <x:c r="F30" s="60" t="n">
+        <x:v>0.002</x:v>
+      </x:c>
+      <x:c r="G30" s="60" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="H30" s="60" t="str">
+        <x:v>analysis_conditions.max_axial_strain</x:v>
+      </x:c>
+      <x:c r="I30" s="60" t="str">
+        <x:v>User editable</x:v>
+      </x:c>
+      <x:c r="J30" s="60" t="str">
+        <x:v>Future tension/bending coupling request.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="15" hidden="0" customHeight="1">
+      <x:c r="A31" s="60" t="str">
+        <x:v>Analysis</x:v>
+      </x:c>
+      <x:c r="B31" s="60" t="str">
+        <x:v>Conditions</x:v>
+      </x:c>
+      <x:c r="C31" s="60" t="str">
+        <x:v>Radial compression ratio</x:v>
+      </x:c>
+      <x:c r="D31" s="60" t="str">
+        <x:v>radial_compression</x:v>
+      </x:c>
+      <x:c r="E31" s="60" t="str">
+        <x:v>QLineEdit</x:v>
+      </x:c>
+      <x:c r="F31" s="60" t="n">
+        <x:v>0.015</x:v>
+      </x:c>
+      <x:c r="G31" s="60" t="str">
+        <x:v>-</x:v>
+      </x:c>
+      <x:c r="H31" s="60" t="str">
+        <x:v>analysis_conditions.radial_compression_ratio</x:v>
+      </x:c>
+      <x:c r="I31" s="60" t="str">
+        <x:v>User editable</x:v>
+      </x:c>
+      <x:c r="J31" s="60" t="str">
+        <x:v>Compression/bird-caging risk request.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="15" hidden="0" customHeight="1">
+      <x:c r="A32" s="60" t="str">
+        <x:v>Analysis</x:v>
+      </x:c>
+      <x:c r="B32" s="60" t="str">
+        <x:v>Conditions</x:v>
+      </x:c>
+      <x:c r="C32" s="60" t="str">
+        <x:v>Loading cycles</x:v>
+      </x:c>
+      <x:c r="D32" s="60" t="str">
+        <x:v>cycles</x:v>
+      </x:c>
+      <x:c r="E32" s="60" t="str">
         <x:v>QSpinBox</x:v>
       </x:c>
-      <x:c r="F28" s="46" t="n">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="G28" s="46" t="str">
+      <x:c r="F32" s="60" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G32" s="60" t="str">
         <x:v>count</x:v>
       </x:c>
-      <x:c r="H28" s="46" t="str">
-        <x:v>mesh.filler_divisions / filler_z_divisions; mesh_controls.Filler.z.count</x:v>
-      </x:c>
-      <x:c r="I28" s="46" t="str">
+      <x:c r="H32" s="60" t="str">
+        <x:v>analysis_conditions.loading_cycles</x:v>
+      </x:c>
+      <x:c r="I32" s="60" t="str">
         <x:v>User editable</x:v>
       </x:c>
-      <x:c r="J28" s="41" t="str">
-        <x:v>Axial divisions for filler special profile.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29" ht="15" hidden="0" customHeight="1">
-      <x:c r="A29" s="40" t="str">
+      <x:c r="J32" s="60" t="str">
+        <x:v>Number of loading cycles in preview/result request.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="15" hidden="0" customHeight="1">
+      <x:c r="A33" s="60" t="str">
         <x:v>Analysis</x:v>
       </x:c>
-      <x:c r="B29" s="46" t="str">
+      <x:c r="B33" s="60" t="str">
         <x:v>Conditions</x:v>
       </x:c>
-      <x:c r="C29" s="46" t="str">
-        <x:v>Effective length</x:v>
-      </x:c>
-      <x:c r="D29" s="46" t="str">
-        <x:v>eff_length</x:v>
-      </x:c>
-      <x:c r="E29" s="46" t="str">
-        <x:v>QLineEdit</x:v>
-      </x:c>
-      <x:c r="F29" s="46" t="n">
-        <x:v>234.2</x:v>
-      </x:c>
-      <x:c r="G29" s="46" t="str">
-        <x:v>mm</x:v>
-      </x:c>
-      <x:c r="H29" s="46" t="str">
-        <x:v>analysis_conditions.effective_length_mm</x:v>
-      </x:c>
-      <x:c r="I29" s="46" t="str">
+      <x:c r="C33" s="60" t="str">
+        <x:v>Result steps</x:v>
+      </x:c>
+      <x:c r="D33" s="60" t="str">
+        <x:v>steps</x:v>
+      </x:c>
+      <x:c r="E33" s="60" t="str">
+        <x:v>QSpinBox</x:v>
+      </x:c>
+      <x:c r="F33" s="60" t="n">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="G33" s="60" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="H33" s="60" t="str">
+        <x:v>analysis_conditions.solver_steps</x:v>
+      </x:c>
+      <x:c r="I33" s="60" t="str">
         <x:v>User editable</x:v>
       </x:c>
-      <x:c r="J29" s="41" t="str">
-        <x:v>Effective length used by backend bending request.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30" ht="15" hidden="0" customHeight="1">
-      <x:c r="A30" s="40" t="str">
-        <x:v>Analysis</x:v>
-      </x:c>
-      <x:c r="B30" s="46" t="str">
-        <x:v>Conditions</x:v>
-      </x:c>
-      <x:c r="C30" s="46" t="str">
-        <x:v>Max twist</x:v>
-      </x:c>
-      <x:c r="D30" s="46" t="str">
-        <x:v>twist</x:v>
-      </x:c>
-      <x:c r="E30" s="46" t="str">
-        <x:v>QLineEdit</x:v>
-      </x:c>
-      <x:c r="F30" s="46" t="n">
-        <x:v>0.05</x:v>
-      </x:c>
-      <x:c r="G30" s="46" t="str">
-        <x:v>rad/m</x:v>
-      </x:c>
-      <x:c r="H30" s="46" t="str">
-        <x:v>analysis_conditions.max_twist_rad_per_m</x:v>
-      </x:c>
-      <x:c r="I30" s="46" t="str">
-        <x:v>User editable</x:v>
-      </x:c>
-      <x:c r="J30" s="41" t="str">
-        <x:v>Future coupled torsion request.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" ht="15" hidden="0" customHeight="1">
-      <x:c r="A31" s="40" t="str">
-        <x:v>Analysis</x:v>
-      </x:c>
-      <x:c r="B31" s="46" t="str">
-        <x:v>Conditions</x:v>
-      </x:c>
-      <x:c r="C31" s="46" t="str">
-        <x:v>Max axial strain</x:v>
-      </x:c>
-      <x:c r="D31" s="46" t="str">
-        <x:v>axial_strain</x:v>
-      </x:c>
-      <x:c r="E31" s="46" t="str">
-        <x:v>QLineEdit</x:v>
-      </x:c>
-      <x:c r="F31" s="46" t="n">
-        <x:v>0.002</x:v>
-      </x:c>
-      <x:c r="G31" s="46" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="H31" s="46" t="str">
-        <x:v>analysis_conditions.max_axial_strain</x:v>
-      </x:c>
-      <x:c r="I31" s="46" t="str">
-        <x:v>User editable</x:v>
-      </x:c>
-      <x:c r="J31" s="41" t="str">
-        <x:v>Future tension/bending coupling request.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32" ht="15" hidden="0" customHeight="1">
-      <x:c r="A32" s="40" t="str">
-        <x:v>Analysis</x:v>
-      </x:c>
-      <x:c r="B32" s="46" t="str">
-        <x:v>Conditions</x:v>
-      </x:c>
-      <x:c r="C32" s="46" t="str">
-        <x:v>Radial compression ratio</x:v>
-      </x:c>
-      <x:c r="D32" s="46" t="str">
-        <x:v>radial_compression</x:v>
-      </x:c>
-      <x:c r="E32" s="46" t="str">
-        <x:v>QLineEdit</x:v>
-      </x:c>
-      <x:c r="F32" s="46" t="n">
-        <x:v>0.015</x:v>
-      </x:c>
-      <x:c r="G32" s="46" t="str">
-        <x:v>-</x:v>
-      </x:c>
-      <x:c r="H32" s="46" t="str">
-        <x:v>analysis_conditions.radial_compression_ratio</x:v>
-      </x:c>
-      <x:c r="I32" s="46" t="str">
-        <x:v>User editable</x:v>
-      </x:c>
-      <x:c r="J32" s="41" t="str">
-        <x:v>Compression/bird-caging risk request.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33" ht="15" hidden="0" customHeight="1">
-      <x:c r="A33" s="40" t="str">
-        <x:v>Analysis</x:v>
-      </x:c>
-      <x:c r="B33" s="46" t="str">
-        <x:v>Conditions</x:v>
-      </x:c>
-      <x:c r="C33" s="46" t="str">
-        <x:v>Loading cycles</x:v>
-      </x:c>
-      <x:c r="D33" s="46" t="str">
-        <x:v>cycles</x:v>
-      </x:c>
-      <x:c r="E33" s="46" t="str">
-        <x:v>QSpinBox</x:v>
-      </x:c>
-      <x:c r="F33" s="46" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G33" s="46" t="str">
-        <x:v>count</x:v>
-      </x:c>
-      <x:c r="H33" s="46" t="str">
-        <x:v>analysis_conditions.loading_cycles</x:v>
-      </x:c>
-      <x:c r="I33" s="46" t="str">
-        <x:v>User editable</x:v>
-      </x:c>
-      <x:c r="J33" s="41" t="str">
-        <x:v>Number of loading cycles in preview/result request.</x:v>
+      <x:c r="J33" s="60" t="str">
+        <x:v>Number of output samples.</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="15" hidden="0" customHeight="1">
-      <x:c r="A34" s="42" t="str">
-        <x:v>Analysis</x:v>
-      </x:c>
-      <x:c r="B34" s="47" t="str">
-        <x:v>Conditions</x:v>
-      </x:c>
-      <x:c r="C34" s="47" t="str">
-        <x:v>Result steps</x:v>
-      </x:c>
-      <x:c r="D34" s="47" t="str">
-        <x:v>steps</x:v>
-      </x:c>
-      <x:c r="E34" s="47" t="str">
-        <x:v>QSpinBox</x:v>
-      </x:c>
-      <x:c r="F34" s="47" t="n">
-        <x:v>500</x:v>
-      </x:c>
-      <x:c r="G34" s="47" t="str">
-        <x:v>count</x:v>
-      </x:c>
-      <x:c r="H34" s="47" t="str">
-        <x:v>analysis_conditions.solver_steps</x:v>
-      </x:c>
-      <x:c r="I34" s="47" t="str">
-        <x:v>User editable</x:v>
-      </x:c>
-      <x:c r="J34" s="43" t="str">
-        <x:v>Number of output samples.</x:v>
-      </x:c>
+      <x:c r="A34" s="42"/>
+      <x:c r="B34" s="47"/>
+      <x:c r="C34" s="47"/>
+      <x:c r="D34" s="47"/>
+      <x:c r="E34" s="47"/>
+      <x:c r="F34" s="47"/>
+      <x:c r="G34" s="47"/>
+      <x:c r="H34" s="47"/>
+      <x:c r="I34" s="47"/>
+      <x:c r="J34" s="43"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2089,13 +2167,13 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="58" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="48" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="72" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="69.37999725341797" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="69.37999725341797" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="69.37999725341797" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="69.37999725341797" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="70.87999725341797" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="69.37999725341797" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="69.37999725341797" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="16.799999237060547" hidden="0" customHeight="1">
@@ -2144,7 +2222,7 @@
         <x:v>Variables not typed directly by the user, but exported or used internally by GUI/backend logic.</x:v>
       </x:c>
     </x:row>
-    <x:row r="3">
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
       <x:c r="A3" s="36"/>
       <x:c r="B3" s="36"/>
       <x:c r="C3" s="36"/>
@@ -2154,439 +2232,554 @@
       <x:c r="G3" s="36"/>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="37" t="str">
+      <x:c r="A4" s="62" t="str">
         <x:v>Variable</x:v>
       </x:c>
-      <x:c r="B4" s="37" t="str">
+      <x:c r="B4" s="62" t="str">
         <x:v>Group</x:v>
       </x:c>
-      <x:c r="C4" s="37" t="str">
+      <x:c r="C4" s="62" t="str">
         <x:v>Formula / Assignment</x:v>
       </x:c>
-      <x:c r="D4" s="37" t="str">
+      <x:c r="D4" s="62" t="str">
         <x:v>Unit</x:v>
       </x:c>
-      <x:c r="E4" s="37" t="str">
+      <x:c r="E4" s="62" t="str">
         <x:v>Payload Path</x:v>
       </x:c>
-      <x:c r="F4" s="37" t="str">
+      <x:c r="F4" s="62" t="str">
         <x:v>Source Type</x:v>
       </x:c>
-      <x:c r="G4" s="37" t="str">
+      <x:c r="G4" s="62" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
-      <x:c r="A5" s="38" t="str">
+      <x:c r="A5" s="60" t="str">
         <x:v>core_center_radius_mm</x:v>
       </x:c>
-      <x:c r="B5" s="45" t="str">
+      <x:c r="B5" s="60" t="str">
         <x:v>Derived geometry</x:v>
       </x:c>
-      <x:c r="C5" s="45" t="str">
+      <x:c r="C5" s="60" t="str">
         <x:v>2*sqrt(3)/3 * core_outer_radius_mm</x:v>
       </x:c>
-      <x:c r="D5" s="45" t="str">
+      <x:c r="D5" s="60" t="str">
         <x:v>mm</x:v>
       </x:c>
-      <x:c r="E5" s="45" t="str">
+      <x:c r="E5" s="60" t="str">
         <x:v>derived_geometry_mm.core_center_radius_mm; geometry_mm.core_center_radius_mm</x:v>
       </x:c>
-      <x:c r="F5" s="45" t="str">
+      <x:c r="F5" s="60" t="str">
         <x:v>Internal auto-derived</x:v>
       </x:c>
-      <x:c r="G5" s="39" t="str">
+      <x:c r="G5" s="60" t="str">
         <x:v>GUI input removed; still exported for backend geometry.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
-      <x:c r="A6" s="40" t="str">
+      <x:c r="A6" s="60" t="str">
         <x:v>inner_sheath_inner_radius_mm</x:v>
       </x:c>
-      <x:c r="B6" s="46" t="str">
+      <x:c r="B6" s="60" t="str">
         <x:v>Derived geometry</x:v>
       </x:c>
-      <x:c r="C6" s="46" t="str">
+      <x:c r="C6" s="60" t="str">
         <x:v>core_outer_radius_mm + core_center_radius_mm</x:v>
       </x:c>
-      <x:c r="D6" s="46" t="str">
+      <x:c r="D6" s="60" t="str">
         <x:v>mm</x:v>
       </x:c>
-      <x:c r="E6" s="46" t="str">
+      <x:c r="E6" s="60" t="str">
         <x:v>derived_geometry_mm.inner_sheath_inner_radius_mm</x:v>
       </x:c>
-      <x:c r="F6" s="46" t="str">
+      <x:c r="F6" s="60" t="str">
         <x:v>Internal auto-derived</x:v>
       </x:c>
-      <x:c r="G6" s="41" t="str">
+      <x:c r="G6" s="60" t="str">
         <x:v>Inner sheath inner radius.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="40" t="str">
+      <x:c r="A7" s="60" t="str">
         <x:v>inner_sheath_outer_radius_mm</x:v>
       </x:c>
-      <x:c r="B7" s="46" t="str">
+      <x:c r="B7" s="60" t="str">
         <x:v>Derived geometry</x:v>
       </x:c>
-      <x:c r="C7" s="46" t="str">
+      <x:c r="C7" s="60" t="str">
         <x:v>inner_sheath_inner_radius_mm + t_is</x:v>
       </x:c>
-      <x:c r="D7" s="46" t="str">
+      <x:c r="D7" s="60" t="str">
         <x:v>mm</x:v>
       </x:c>
-      <x:c r="E7" s="46" t="str">
+      <x:c r="E7" s="60" t="str">
         <x:v>derived_geometry_mm.inner_sheath_outer_radius_mm</x:v>
       </x:c>
-      <x:c r="F7" s="46" t="str">
+      <x:c r="F7" s="60" t="str">
         <x:v>Internal auto-derived</x:v>
       </x:c>
-      <x:c r="G7" s="41" t="str">
+      <x:c r="G7" s="60" t="str">
         <x:v>Inner sheath outer radius.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
-      <x:c r="A8" s="40" t="str">
+      <x:c r="A8" s="60" t="str">
         <x:v>inner_armour_center_radius_mm</x:v>
       </x:c>
-      <x:c r="B8" s="46" t="str">
+      <x:c r="B8" s="60" t="str">
         <x:v>Derived geometry</x:v>
       </x:c>
-      <x:c r="C8" s="46" t="str">
+      <x:c r="C8" s="60" t="str">
         <x:v>inner_sheath_outer_radius_mm + r_ia</x:v>
       </x:c>
-      <x:c r="D8" s="46" t="str">
+      <x:c r="D8" s="60" t="str">
         <x:v>mm</x:v>
       </x:c>
-      <x:c r="E8" s="46" t="str">
+      <x:c r="E8" s="60" t="str">
         <x:v>derived_geometry_mm.inner_armour_center_radius_mm</x:v>
       </x:c>
-      <x:c r="F8" s="46" t="str">
+      <x:c r="F8" s="60" t="str">
         <x:v>Internal auto-derived</x:v>
       </x:c>
-      <x:c r="G8" s="41" t="str">
+      <x:c r="G8" s="60" t="str">
         <x:v>Assumes clearance gap = 0.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
-      <x:c r="A9" s="40" t="str">
+      <x:c r="A9" s="60" t="str">
         <x:v>inner_armour_outer_radius_mm</x:v>
       </x:c>
-      <x:c r="B9" s="46" t="str">
+      <x:c r="B9" s="60" t="str">
         <x:v>Derived geometry</x:v>
       </x:c>
-      <x:c r="C9" s="46" t="str">
+      <x:c r="C9" s="60" t="str">
         <x:v>inner_armour_center_radius_mm + r_ia</x:v>
       </x:c>
-      <x:c r="D9" s="46" t="str">
+      <x:c r="D9" s="60" t="str">
         <x:v>mm</x:v>
       </x:c>
-      <x:c r="E9" s="46" t="str">
+      <x:c r="E9" s="60" t="str">
         <x:v>derived_geometry_mm.inner_armour_outer_radius_mm</x:v>
       </x:c>
-      <x:c r="F9" s="46" t="str">
+      <x:c r="F9" s="60" t="str">
         <x:v>Internal auto-derived</x:v>
       </x:c>
-      <x:c r="G9" s="41" t="str">
+      <x:c r="G9" s="60" t="str">
         <x:v>Outer radius of inner armour envelope.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
-      <x:c r="A10" s="40" t="str">
+      <x:c r="A10" s="60" t="str">
         <x:v>bedding_outer_radius_mm</x:v>
       </x:c>
-      <x:c r="B10" s="46" t="str">
+      <x:c r="B10" s="60" t="str">
         <x:v>Derived geometry</x:v>
       </x:c>
-      <x:c r="C10" s="46" t="str">
+      <x:c r="C10" s="60" t="str">
         <x:v>inner_armour_outer_radius_mm + bedding_thickness</x:v>
       </x:c>
-      <x:c r="D10" s="46" t="str">
+      <x:c r="D10" s="60" t="str">
         <x:v>mm</x:v>
       </x:c>
-      <x:c r="E10" s="46" t="str">
+      <x:c r="E10" s="60" t="str">
         <x:v>derived_geometry_mm.bedding_outer_radius_mm</x:v>
       </x:c>
-      <x:c r="F10" s="46" t="str">
+      <x:c r="F10" s="60" t="str">
         <x:v>Internal auto-derived</x:v>
       </x:c>
-      <x:c r="G10" s="41" t="str">
+      <x:c r="G10" s="60" t="str">
         <x:v>Bedding outer radius.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
-      <x:c r="A11" s="40" t="str">
+      <x:c r="A11" s="60" t="str">
         <x:v>outer_armour_center_radius_mm</x:v>
       </x:c>
-      <x:c r="B11" s="46" t="str">
+      <x:c r="B11" s="60" t="str">
         <x:v>Derived geometry</x:v>
       </x:c>
-      <x:c r="C11" s="46" t="str">
+      <x:c r="C11" s="60" t="str">
         <x:v>bedding_outer_radius_mm + r_oa</x:v>
       </x:c>
-      <x:c r="D11" s="46" t="str">
+      <x:c r="D11" s="60" t="str">
         <x:v>mm</x:v>
       </x:c>
-      <x:c r="E11" s="46" t="str">
+      <x:c r="E11" s="60" t="str">
         <x:v>derived_geometry_mm.outer_armour_center_radius_mm</x:v>
       </x:c>
-      <x:c r="F11" s="46" t="str">
+      <x:c r="F11" s="60" t="str">
         <x:v>Internal auto-derived</x:v>
       </x:c>
-      <x:c r="G11" s="41" t="str">
+      <x:c r="G11" s="60" t="str">
         <x:v>Assumes clearance gap = 0.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
-      <x:c r="A12" s="40" t="str">
+      <x:c r="A12" s="60" t="str">
         <x:v>outer_sheath_inner_radius_mm</x:v>
       </x:c>
-      <x:c r="B12" s="46" t="str">
+      <x:c r="B12" s="60" t="str">
         <x:v>Derived geometry</x:v>
       </x:c>
-      <x:c r="C12" s="46" t="str">
+      <x:c r="C12" s="60" t="str">
         <x:v>outer_armour_center_radius_mm + r_oa</x:v>
       </x:c>
-      <x:c r="D12" s="46" t="str">
+      <x:c r="D12" s="60" t="str">
         <x:v>mm</x:v>
       </x:c>
-      <x:c r="E12" s="46" t="str">
+      <x:c r="E12" s="60" t="str">
         <x:v>derived_geometry_mm.outer_sheath_inner_radius_mm</x:v>
       </x:c>
-      <x:c r="F12" s="46" t="str">
+      <x:c r="F12" s="60" t="str">
         <x:v>Internal auto-derived</x:v>
       </x:c>
-      <x:c r="G12" s="41" t="str">
+      <x:c r="G12" s="60" t="str">
         <x:v>Outer sheath inner radius.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
-      <x:c r="A13" s="40" t="str">
+      <x:c r="A13" s="60" t="str">
         <x:v>outer_sheath_outer_radius_mm</x:v>
       </x:c>
-      <x:c r="B13" s="46" t="str">
+      <x:c r="B13" s="60" t="str">
         <x:v>Derived geometry</x:v>
       </x:c>
-      <x:c r="C13" s="46" t="str">
+      <x:c r="C13" s="60" t="str">
         <x:v>outer_sheath_inner_radius_mm + t_os</x:v>
       </x:c>
-      <x:c r="D13" s="46" t="str">
+      <x:c r="D13" s="60" t="str">
         <x:v>mm</x:v>
       </x:c>
-      <x:c r="E13" s="46" t="str">
+      <x:c r="E13" s="60" t="str">
         <x:v>derived_geometry_mm.outer_sheath_outer_radius_mm</x:v>
       </x:c>
-      <x:c r="F13" s="46" t="str">
+      <x:c r="F13" s="60" t="str">
         <x:v>Internal auto-derived</x:v>
       </x:c>
-      <x:c r="G13" s="41" t="str">
+      <x:c r="G13" s="60" t="str">
         <x:v>Cable outer radius in preview.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
-      <x:c r="A14" s="40" t="str">
+      <x:c r="A14" s="60" t="str">
+        <x:v>core_pitch_length_mm</x:v>
+      </x:c>
+      <x:c r="B14" s="60" t="str">
+        <x:v>Derived pitch</x:v>
+      </x:c>
+      <x:c r="C14" s="60" t="str">
+        <x:v>2*pi*core_center_radius_mm/tan(core_lay_angle_deg)</x:v>
+      </x:c>
+      <x:c r="D14" s="60" t="str">
+        <x:v>mm</x:v>
+      </x:c>
+      <x:c r="E14" s="60" t="str">
+        <x:v>derived_geometry_mm.core_pitch_length_mm; armour.core_pitch_length_mm</x:v>
+      </x:c>
+      <x:c r="F14" s="60" t="str">
+        <x:v>Internal auto-derived</x:v>
+      </x:c>
+      <x:c r="G14" s="60" t="str">
+        <x:v>Displayed in Design tab and used for effective length.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="15" hidden="0" customHeight="1">
+      <x:c r="A15" s="60" t="str">
+        <x:v>inner_armour_pitch_length_mm</x:v>
+      </x:c>
+      <x:c r="B15" s="60" t="str">
+        <x:v>Derived pitch</x:v>
+      </x:c>
+      <x:c r="C15" s="60" t="str">
+        <x:v>2*pi*inner_armour_center_radius_mm/tan(inner_armour_lay_angle_deg)</x:v>
+      </x:c>
+      <x:c r="D15" s="60" t="str">
+        <x:v>mm</x:v>
+      </x:c>
+      <x:c r="E15" s="60" t="str">
+        <x:v>derived_geometry_mm.inner_armour_pitch_length_mm; armour.inner_armour_pitch_length_mm</x:v>
+      </x:c>
+      <x:c r="F15" s="60" t="str">
+        <x:v>Internal auto-derived</x:v>
+      </x:c>
+      <x:c r="G15" s="60" t="str">
+        <x:v>Positive pitch length; signed pitch is also exported for Abaqus compatibility.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="15" hidden="0" customHeight="1">
+      <x:c r="A16" s="60" t="str">
+        <x:v>outer_armour_pitch_length_mm</x:v>
+      </x:c>
+      <x:c r="B16" s="60" t="str">
+        <x:v>Derived pitch</x:v>
+      </x:c>
+      <x:c r="C16" s="60" t="str">
+        <x:v>2*pi*outer_armour_center_radius_mm/tan(outer_armour_lay_angle_deg)</x:v>
+      </x:c>
+      <x:c r="D16" s="60" t="str">
+        <x:v>mm</x:v>
+      </x:c>
+      <x:c r="E16" s="60" t="str">
+        <x:v>derived_geometry_mm.outer_armour_pitch_length_mm; armour.outer_armour_pitch_length_mm</x:v>
+      </x:c>
+      <x:c r="F16" s="60" t="str">
+        <x:v>Internal auto-derived</x:v>
+      </x:c>
+      <x:c r="G16" s="60" t="str">
+        <x:v>Positive pitch length; signed pitch is also exported for Abaqus compatibility.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="15" hidden="0" customHeight="1">
+      <x:c r="A17" s="60" t="str">
+        <x:v>effective_length_mm</x:v>
+      </x:c>
+      <x:c r="B17" s="60" t="str">
+        <x:v>Derived analysis length</x:v>
+      </x:c>
+      <x:c r="C17" s="60" t="str">
+        <x:v>core_pitch_length_mm / core_count</x:v>
+      </x:c>
+      <x:c r="D17" s="60" t="str">
+        <x:v>mm</x:v>
+      </x:c>
+      <x:c r="E17" s="60" t="str">
+        <x:v>analysis_conditions.effective_length_mm; derived_geometry_mm.effective_length_mm</x:v>
+      </x:c>
+      <x:c r="F17" s="60" t="str">
+        <x:v>Read-only derived display</x:v>
+      </x:c>
+      <x:c r="G17" s="60" t="str">
+        <x:v>No longer user editable; Analysis tab displays the computed value.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
+      <x:c r="A18" s="60" t="str">
+        <x:v>filler_z_divisions</x:v>
+      </x:c>
+      <x:c r="B18" s="60" t="str">
+        <x:v>Mesh compatibility mirror</x:v>
+      </x:c>
+      <x:c r="C18" s="60" t="str">
+        <x:v>mesh.axial_divisions</x:v>
+      </x:c>
+      <x:c r="D18" s="60" t="str">
+        <x:v>count</x:v>
+      </x:c>
+      <x:c r="E18" s="60" t="str">
+        <x:v>mesh.filler_z_divisions; mesh.filler_divisions</x:v>
+      </x:c>
+      <x:c r="F18" s="60" t="str">
+        <x:v>Internal compatibility key</x:v>
+      </x:c>
+      <x:c r="G18" s="60" t="str">
+        <x:v>No separate GUI input; source is same_as_axial_divisions.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="15" hidden="0" customHeight="1">
+      <x:c r="A19" s="60" t="str">
         <x:v>inner_armour_wire_count_limit</x:v>
       </x:c>
-      <x:c r="B14" s="46" t="str">
+      <x:c r="B19" s="60" t="str">
         <x:v>Derived count</x:v>
       </x:c>
-      <x:c r="C14" s="46" t="str">
+      <x:c r="C19" s="60" t="str">
         <x:v>floor(pi/asin(r_ia/R_inner_armour_center))</x:v>
       </x:c>
-      <x:c r="D14" s="46" t="str">
+      <x:c r="D19" s="60" t="str">
         <x:v>count</x:v>
       </x:c>
-      <x:c r="E14" s="46" t="str">
+      <x:c r="E19" s="60" t="str">
         <x:v>derived_geometry_mm.inner_armour_wire_count_limit</x:v>
       </x:c>
-      <x:c r="F14" s="46" t="str">
+      <x:c r="F19" s="60" t="str">
         <x:v>Internal limit/clamp</x:v>
       </x:c>
-      <x:c r="G14" s="41" t="str">
+      <x:c r="G19" s="60" t="str">
         <x:v>SpinBox maximum; prevents physically impossible count.</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="15" hidden="0" customHeight="1">
-      <x:c r="A15" s="40" t="str">
+    <x:row r="20" ht="15" hidden="0" customHeight="1">
+      <x:c r="A20" s="60" t="str">
         <x:v>outer_armour_wire_count_limit</x:v>
       </x:c>
-      <x:c r="B15" s="46" t="str">
+      <x:c r="B20" s="60" t="str">
         <x:v>Derived count</x:v>
       </x:c>
-      <x:c r="C15" s="46" t="str">
+      <x:c r="C20" s="60" t="str">
         <x:v>floor(pi/asin(r_oa/R_outer_armour_center))</x:v>
       </x:c>
-      <x:c r="D15" s="46" t="str">
+      <x:c r="D20" s="60" t="str">
         <x:v>count</x:v>
       </x:c>
-      <x:c r="E15" s="46" t="str">
+      <x:c r="E20" s="60" t="str">
         <x:v>derived_geometry_mm.outer_armour_wire_count_limit</x:v>
       </x:c>
-      <x:c r="F15" s="46" t="str">
+      <x:c r="F20" s="60" t="str">
         <x:v>Internal limit/clamp</x:v>
       </x:c>
-      <x:c r="G15" s="41" t="str">
+      <x:c r="G20" s="60" t="str">
         <x:v>SpinBox maximum; prevents physically impossible count.</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="15" hidden="0" customHeight="1">
-      <x:c r="A16" s="40" t="str">
+    <x:row r="21" ht="15" hidden="0" customHeight="1">
+      <x:c r="A21" s="60" t="str">
         <x:v>inner_wire_count_resolved</x:v>
       </x:c>
-      <x:c r="B16" s="46" t="str">
+      <x:c r="B21" s="60" t="str">
         <x:v>Derived count</x:v>
       </x:c>
-      <x:c r="C16" s="46" t="str">
+      <x:c r="C21" s="60" t="str">
         <x:v>user no_ia if &gt;0 else formula limit</x:v>
       </x:c>
-      <x:c r="D16" s="46" t="str">
+      <x:c r="D21" s="60" t="str">
         <x:v>count</x:v>
       </x:c>
-      <x:c r="E16" s="46" t="str">
+      <x:c r="E21" s="60" t="str">
         <x:v>armour.inner_wire_count_resolved</x:v>
       </x:c>
-      <x:c r="F16" s="46" t="str">
+      <x:c r="F21" s="60" t="str">
         <x:v>Internal resolution</x:v>
       </x:c>
-      <x:c r="G16" s="41" t="str">
+      <x:c r="G21" s="60" t="str">
         <x:v>Backend uses resolved count.</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="15" hidden="0" customHeight="1">
-      <x:c r="A17" s="40" t="str">
+    <x:row r="22" ht="15" hidden="0" customHeight="1">
+      <x:c r="A22" s="60" t="str">
         <x:v>outer_wire_count_resolved</x:v>
       </x:c>
-      <x:c r="B17" s="46" t="str">
+      <x:c r="B22" s="60" t="str">
         <x:v>Derived count</x:v>
       </x:c>
-      <x:c r="C17" s="46" t="str">
+      <x:c r="C22" s="60" t="str">
         <x:v>user no_oa if &gt;0 else formula limit</x:v>
       </x:c>
-      <x:c r="D17" s="46" t="str">
+      <x:c r="D22" s="60" t="str">
         <x:v>count</x:v>
       </x:c>
-      <x:c r="E17" s="46" t="str">
+      <x:c r="E22" s="60" t="str">
         <x:v>armour.outer_wire_count_resolved</x:v>
       </x:c>
-      <x:c r="F17" s="46" t="str">
+      <x:c r="F22" s="60" t="str">
         <x:v>Internal resolution</x:v>
       </x:c>
-      <x:c r="G17" s="41" t="str">
+      <x:c r="G22" s="60" t="str">
         <x:v>Backend uses resolved count.</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="15" hidden="0" customHeight="1">
-      <x:c r="A18" s="40" t="str">
+    <x:row r="23" ht="15" hidden="0" customHeight="1">
+      <x:c r="A23" s="68" t="str">
         <x:v>clearance_gap_mm</x:v>
       </x:c>
-      <x:c r="B18" s="46" t="str">
+      <x:c r="B23" s="68" t="str">
         <x:v>Fixed internal geometry</x:v>
       </x:c>
-      <x:c r="C18" s="46" t="str">
+      <x:c r="C23" s="68" t="str">
         <x:v>0.0</x:v>
       </x:c>
-      <x:c r="D18" s="46" t="str">
+      <x:c r="D23" s="68" t="str">
         <x:v>mm</x:v>
       </x:c>
-      <x:c r="E18" s="46" t="str">
+      <x:c r="E23" s="68" t="str">
         <x:v>geometry_mm.clearance_gap_mm; derived_geometry_mm.clearance_gap_mm</x:v>
       </x:c>
-      <x:c r="F18" s="46" t="str">
+      <x:c r="F23" s="68" t="str">
         <x:v>Fixed internal default</x:v>
       </x:c>
-      <x:c r="G18" s="41" t="str">
+      <x:c r="G23" s="68" t="str">
         <x:v>GUI input removed; current design treats gap as zero.</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="15" hidden="0" customHeight="1">
-      <x:c r="A19" s="40" t="str">
+    <x:row r="24" ht="15" hidden="0" customHeight="1">
+      <x:c r="A24" s="68" t="str">
         <x:v>filler_count</x:v>
       </x:c>
-      <x:c r="B19" s="46" t="str">
+      <x:c r="B24" s="68" t="str">
         <x:v>Fixed internal geometry</x:v>
       </x:c>
-      <x:c r="C19" s="46" t="str">
+      <x:c r="C24" s="68" t="str">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="D19" s="46" t="str">
+      <x:c r="D24" s="68" t="str">
         <x:v>count</x:v>
       </x:c>
-      <x:c r="E19" s="46" t="str">
+      <x:c r="E24" s="68" t="str">
         <x:v>derived_geometry_mm.filler_count</x:v>
       </x:c>
-      <x:c r="F19" s="46" t="str">
+      <x:c r="F24" s="68" t="str">
         <x:v>Fixed internal default</x:v>
       </x:c>
-      <x:c r="G19" s="41" t="str">
+      <x:c r="G24" s="68" t="str">
         <x:v>Three filler regions in current section model.</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="15" hidden="0" customHeight="1">
-      <x:c r="A20" s="40" t="str">
+    <x:row r="25" ht="15" hidden="0" customHeight="1">
+      <x:c r="A25" s="68" t="str">
         <x:v>filler_profile_scale</x:v>
       </x:c>
-      <x:c r="B20" s="46" t="str">
+      <x:c r="B25" s="68" t="str">
         <x:v>Derived geometry</x:v>
       </x:c>
-      <x:c r="C20" s="46" t="str">
+      <x:c r="C25" s="68" t="str">
         <x:v>core_outer_radius_mm / 15.3</x:v>
       </x:c>
-      <x:c r="D20" s="46" t="str">
+      <x:c r="D25" s="68" t="str">
         <x:v>-</x:v>
       </x:c>
-      <x:c r="E20" s="46" t="str">
+      <x:c r="E25" s="68" t="str">
         <x:v>derived_geometry_mm.filler_profile_scale</x:v>
       </x:c>
-      <x:c r="F20" s="46" t="str">
+      <x:c r="F25" s="68" t="str">
         <x:v>Internal auto-derived</x:v>
       </x:c>
-      <x:c r="G20" s="41" t="str">
+      <x:c r="G25" s="68" t="str">
         <x:v>Scales filler sketch/profile with core outer radius.</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="15" hidden="0" customHeight="1">
-      <x:c r="A21" s="40" t="str">
+    <x:row r="26" ht="15" hidden="0" customHeight="1">
+      <x:c r="A26" s="68" t="str">
         <x:v>lay_angle_deg</x:v>
       </x:c>
-      <x:c r="B21" s="46" t="str">
+      <x:c r="B26" s="68" t="str">
         <x:v>Derived armour summary</x:v>
       </x:c>
-      <x:c r="C21" s="46" t="str">
+      <x:c r="C26" s="68" t="str">
         <x:v>0.5*(inner_lay_angle_deg + outer_lay_angle_deg)</x:v>
       </x:c>
-      <x:c r="D21" s="46" t="str">
+      <x:c r="D26" s="68" t="str">
         <x:v>deg</x:v>
       </x:c>
-      <x:c r="E21" s="46" t="str">
+      <x:c r="E26" s="68" t="str">
         <x:v>armour.lay_angle_deg</x:v>
       </x:c>
-      <x:c r="F21" s="46" t="str">
+      <x:c r="F26" s="68" t="str">
         <x:v>Internal summary</x:v>
       </x:c>
-      <x:c r="G21" s="41" t="str">
+      <x:c r="G26" s="68" t="str">
         <x:v>Average armour lay angle kept for backend compatibility.</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="15" hidden="0" customHeight="1">
-      <x:c r="A22" s="42" t="str">
+    <x:row r="27" ht="15" hidden="0" customHeight="1">
+      <x:c r="A27" s="68" t="str">
         <x:v>core_equivalent_EI_N_m2</x:v>
       </x:c>
-      <x:c r="B22" s="47" t="str">
+      <x:c r="B27" s="68" t="str">
         <x:v>GUI estimate</x:v>
       </x:c>
-      <x:c r="C22" s="47" t="str">
-        <x:v>3 conductor cores with parallel axis estimate</x:v>
-      </x:c>
-      <x:c r="D22" s="47" t="str">
+      <x:c r="C27" s="68" t="str">
+        <x:v>core_count conductor cores with parallel axis estimate</x:v>
+      </x:c>
+      <x:c r="D27" s="68" t="str">
         <x:v>N*m^2</x:v>
       </x:c>
-      <x:c r="E22" s="47" t="str">
+      <x:c r="E27" s="68" t="str">
         <x:v>equivalent_properties.core_equivalent_EI_N_m2</x:v>
       </x:c>
-      <x:c r="F22" s="47" t="str">
+      <x:c r="F27" s="68" t="str">
         <x:v>Internal estimate only</x:v>
       </x:c>
-      <x:c r="G22" s="43" t="str">
+      <x:c r="G27" s="68" t="str">
         <x:v>Abaqus result remains authoritative.</x:v>
       </x:c>
     </x:row>
@@ -2603,11 +2796,11 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="46" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="34" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="80" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="57.630001068115234" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="56" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="79.62999725341797" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="56" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="58.5" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="16.799999237060547" hidden="0" customHeight="1">
@@ -2644,7 +2837,7 @@
         <x:v>Constants, hidden defaults, or generated values included in input_data.json.</x:v>
       </x:c>
     </x:row>
-    <x:row r="3">
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
       <x:c r="A3" s="36"/>
       <x:c r="B3" s="36"/>
       <x:c r="C3" s="36"/>
@@ -2652,479 +2845,598 @@
       <x:c r="E3" s="36"/>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="37" t="str">
+      <x:c r="A4" s="62" t="str">
         <x:v>Payload Path</x:v>
       </x:c>
-      <x:c r="B4" s="37" t="str">
+      <x:c r="B4" s="62" t="str">
         <x:v>Code Source</x:v>
       </x:c>
-      <x:c r="C4" s="37" t="str">
+      <x:c r="C4" s="62" t="str">
         <x:v>Default / Value</x:v>
       </x:c>
-      <x:c r="D4" s="37" t="str">
+      <x:c r="D4" s="62" t="str">
         <x:v>Source Type</x:v>
       </x:c>
-      <x:c r="E4" s="37" t="str">
+      <x:c r="E4" s="62" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
-      <x:c r="A5" s="38" t="str">
+      <x:c r="A5" s="60" t="str">
         <x:v>metadata.contract_version</x:v>
       </x:c>
-      <x:c r="B5" s="45" t="str">
+      <x:c r="B5" s="60" t="str">
         <x:v>CONTRACT_VERSION</x:v>
       </x:c>
-      <x:c r="C5" s="45" t="str">
+      <x:c r="C5" s="60" t="str">
         <x:v>sclas-abaqus-contract-v1</x:v>
       </x:c>
-      <x:c r="D5" s="45" t="str">
+      <x:c r="D5" s="60" t="str">
         <x:v>Fixed metadata</x:v>
       </x:c>
-      <x:c r="E5" s="39" t="str">
+      <x:c r="E5" s="60" t="str">
         <x:v>Backend contract version.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
-      <x:c r="A6" s="40" t="str">
+      <x:c r="A6" s="60" t="str">
         <x:v>metadata.frontend_version</x:v>
       </x:c>
-      <x:c r="B6" s="46" t="str">
+      <x:c r="B6" s="60" t="str">
         <x:v>APP_VERSION</x:v>
       </x:c>
-      <x:c r="C6" s="46" t="str">
+      <x:c r="C6" s="60" t="str">
         <x:v>12.0-abaqus-quality-summary</x:v>
       </x:c>
-      <x:c r="D6" s="46" t="str">
+      <x:c r="D6" s="60" t="str">
         <x:v>Fixed metadata</x:v>
       </x:c>
-      <x:c r="E6" s="41" t="str">
+      <x:c r="E6" s="60" t="str">
         <x:v>GUI/frontend version string.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="40" t="str">
+      <x:c r="A7" s="60" t="str">
         <x:v>metadata.job_id</x:v>
       </x:c>
-      <x:c r="B7" s="46" t="str">
+      <x:c r="B7" s="60" t="str">
         <x:v>now_job_id()</x:v>
       </x:c>
-      <x:c r="C7" s="46" t="str">
+      <x:c r="C7" s="60" t="str">
         <x:v>timestamp_uuid</x:v>
       </x:c>
-      <x:c r="D7" s="46" t="str">
+      <x:c r="D7" s="60" t="str">
         <x:v>Generated per run</x:v>
       </x:c>
-      <x:c r="E7" s="41" t="str">
+      <x:c r="E7" s="60" t="str">
         <x:v>Unique job folder id.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
-      <x:c r="A8" s="40" t="str">
+      <x:c r="A8" s="60" t="str">
         <x:v>mesh.model_strategy</x:v>
       </x:c>
-      <x:c r="B8" s="46" t="str">
+      <x:c r="B8" s="60" t="str">
         <x:v>mesh_value('model_strategy')</x:v>
       </x:c>
-      <x:c r="C8" s="46" t="str">
+      <x:c r="C8" s="60" t="str">
         <x:v>full_3d_segment</x:v>
       </x:c>
-      <x:c r="D8" s="46" t="str">
+      <x:c r="D8" s="60" t="str">
         <x:v>Fixed backend default</x:v>
       </x:c>
-      <x:c r="E8" s="41" t="str">
+      <x:c r="E8" s="60" t="str">
         <x:v>Strategy selector removed from visible GUI.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
-      <x:c r="A9" s="40" t="str">
+      <x:c r="A9" s="60" t="str">
         <x:v>mesh.armour_model</x:v>
       </x:c>
-      <x:c r="B9" s="46" t="str">
+      <x:c r="B9" s="60" t="str">
         <x:v>mesh_value('armour_model')</x:v>
       </x:c>
-      <x:c r="C9" s="46" t="str">
+      <x:c r="C9" s="60" t="str">
         <x:v>solid_wire</x:v>
       </x:c>
-      <x:c r="D9" s="46" t="str">
+      <x:c r="D9" s="60" t="str">
         <x:v>Fixed backend default</x:v>
       </x:c>
-      <x:c r="E9" s="41" t="str">
+      <x:c r="E9" s="60" t="str">
         <x:v>Armour model selector removed from visible GUI.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
-      <x:c r="A10" s="40" t="str">
+      <x:c r="A10" s="60" t="str">
         <x:v>mesh.contact_regularization_beta</x:v>
       </x:c>
-      <x:c r="B10" s="46" t="str">
+      <x:c r="B10" s="60" t="str">
         <x:v>contact_beta hidden widget</x:v>
       </x:c>
-      <x:c r="C10" s="46" t="n">
+      <x:c r="C10" s="60" t="n">
         <x:v>0.001</x:v>
       </x:c>
-      <x:c r="D10" s="46" t="str">
+      <x:c r="D10" s="60" t="str">
         <x:v>Hidden GUI/internal</x:v>
       </x:c>
-      <x:c r="E10" s="41" t="str">
+      <x:c r="E10" s="60" t="str">
         <x:v>Tangential contact regularization value.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
-      <x:c r="A11" s="40" t="str">
+      <x:c r="A11" s="60" t="str">
         <x:v>mesh.coordinate_basis</x:v>
       </x:c>
-      <x:c r="B11" s="46" t="str">
+      <x:c r="B11" s="60" t="str">
         <x:v>literal</x:v>
       </x:c>
-      <x:c r="C11" s="46" t="str">
+      <x:c r="C11" s="60" t="str">
         <x:v>cylindrical_r_theta_z</x:v>
       </x:c>
-      <x:c r="D11" s="46" t="str">
+      <x:c r="D11" s="60" t="str">
         <x:v>Fixed backend default</x:v>
       </x:c>
-      <x:c r="E11" s="41" t="str">
+      <x:c r="E11" s="60" t="str">
         <x:v>Coordinate basis for mesh controls.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
-      <x:c r="A12" s="40" t="str">
+      <x:c r="A12" s="60" t="str">
+        <x:v>mesh.axial_divisions_scope</x:v>
+      </x:c>
+      <x:c r="B12" s="60" t="str">
+        <x:v>literal</x:v>
+      </x:c>
+      <x:c r="C12" s="60" t="str">
+        <x:v>global_all_components</x:v>
+      </x:c>
+      <x:c r="D12" s="60" t="str">
+        <x:v>Fixed backend contract</x:v>
+      </x:c>
+      <x:c r="E12" s="60" t="str">
+        <x:v>One global axial n_z count applies to every component.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
+      <x:c r="A13" s="60" t="str">
+        <x:v>mesh.filler_z_divisions_source</x:v>
+      </x:c>
+      <x:c r="B13" s="60" t="str">
+        <x:v>literal</x:v>
+      </x:c>
+      <x:c r="C13" s="60" t="str">
+        <x:v>same_as_axial_divisions</x:v>
+      </x:c>
+      <x:c r="D13" s="60" t="str">
+        <x:v>Fixed backend contract</x:v>
+      </x:c>
+      <x:c r="E13" s="60" t="str">
+        <x:v>Filler z divisions mirror mesh.axial_divisions.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="15" hidden="0" customHeight="1">
+      <x:c r="A14" s="60" t="str">
+        <x:v>analysis_conditions.effective_length_source</x:v>
+      </x:c>
+      <x:c r="B14" s="60" t="str">
+        <x:v>derived geometry</x:v>
+      </x:c>
+      <x:c r="C14" s="60" t="str">
+        <x:v>core_pitch_length_mm_divided_by_core_count</x:v>
+      </x:c>
+      <x:c r="D14" s="60" t="str">
+        <x:v>Fixed derived policy</x:v>
+      </x:c>
+      <x:c r="E14" s="60" t="str">
+        <x:v>Explains why effective_length_mm is read-only in the GUI.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="15" hidden="0" customHeight="1">
+      <x:c r="A15" s="60" t="str">
         <x:v>analysis_conditions.residual_contact_pressure_mpa</x:v>
       </x:c>
-      <x:c r="B12" s="46" t="str">
+      <x:c r="B15" s="60" t="str">
         <x:v>residual_contact_pressure hidden widget</x:v>
       </x:c>
-      <x:c r="C12" s="46" t="n">
+      <x:c r="C15" s="60" t="n">
         <x:v>0.3</x:v>
       </x:c>
-      <x:c r="D12" s="46" t="str">
+      <x:c r="D15" s="60" t="str">
         <x:v>Hidden GUI/internal</x:v>
       </x:c>
-      <x:c r="E12" s="41" t="str">
+      <x:c r="E15" s="60" t="str">
         <x:v>Residual normal contact pressure; hidden from current GUI.</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="15" hidden="0" customHeight="1">
-      <x:c r="A13" s="40" t="str">
+    <x:row r="16" ht="15" hidden="0" customHeight="1">
+      <x:c r="A16" s="60" t="str">
         <x:v>analysis_conditions.curve_factors</x:v>
       </x:c>
-      <x:c r="B13" s="46" t="str">
+      <x:c r="B16" s="60" t="str">
         <x:v>literal</x:v>
       </x:c>
-      <x:c r="C13" s="46" t="str">
+      <x:c r="C16" s="60" t="str">
         <x:v>[-0.1,-0.05,0,0.05,0.1]</x:v>
       </x:c>
-      <x:c r="D13" s="46" t="str">
+      <x:c r="D16" s="60" t="str">
         <x:v>Fixed backend default</x:v>
       </x:c>
-      <x:c r="E13" s="41" t="str">
+      <x:c r="E16" s="60" t="str">
         <x:v>Curve endpoint factors for sweep/CurveV0 style requests.</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="15" hidden="0" customHeight="1">
-      <x:c r="A14" s="40" t="str">
+    <x:row r="17" ht="15" hidden="0" customHeight="1">
+      <x:c r="A17" s="60" t="str">
         <x:v>analysis_conditions.run_mode</x:v>
       </x:c>
-      <x:c r="B14" s="46" t="str">
+      <x:c r="B17" s="60" t="str">
         <x:v>literal</x:v>
       </x:c>
-      <x:c r="C14" s="46" t="str">
+      <x:c r="C17" s="60" t="str">
         <x:v>export_job_only</x:v>
       </x:c>
-      <x:c r="D14" s="46" t="str">
+      <x:c r="D17" s="60" t="str">
         <x:v>Fixed backend default</x:v>
       </x:c>
-      <x:c r="E14" s="41" t="str">
+      <x:c r="E17" s="60" t="str">
         <x:v>Initial package mode; actual runner selection controlled by GUI backend mode.</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="15" hidden="0" customHeight="1">
-      <x:c r="A15" s="40" t="str">
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
+      <x:c r="A18" s="60" t="str">
         <x:v>analysis_conditions.save_abaqus_files</x:v>
       </x:c>
-      <x:c r="B15" s="46" t="str">
+      <x:c r="B18" s="60" t="str">
         <x:v>literal</x:v>
       </x:c>
-      <x:c r="C15" s="51" t="b">
+      <x:c r="C18" s="70" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D15" s="46" t="str">
+      <x:c r="D18" s="60" t="str">
         <x:v>Fixed backend default</x:v>
       </x:c>
-      <x:c r="E15" s="41" t="str">
+      <x:c r="E18" s="60" t="str">
         <x:v>Request Abaqus file generation.</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="15" hidden="0" customHeight="1">
-      <x:c r="A16" s="40" t="str">
+    <x:row r="19" ht="15" hidden="0" customHeight="1">
+      <x:c r="A19" s="60" t="str">
         <x:v>analysis_conditions.run_solver</x:v>
       </x:c>
-      <x:c r="B16" s="46" t="str">
+      <x:c r="B19" s="60" t="str">
         <x:v>literal</x:v>
       </x:c>
-      <x:c r="C16" s="51" t="b">
+      <x:c r="C19" s="70" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D16" s="46" t="str">
+      <x:c r="D19" s="60" t="str">
         <x:v>Fixed backend default</x:v>
       </x:c>
-      <x:c r="E16" s="41" t="str">
+      <x:c r="E19" s="60" t="str">
         <x:v>One-click runner may override execution path; payload default is false.</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="15" hidden="0" customHeight="1">
-      <x:c r="A17" s="40" t="str">
+    <x:row r="20" ht="15" hidden="0" customHeight="1">
+      <x:c r="A20" s="60" t="str">
         <x:v>analysis_conditions.extract_odb</x:v>
       </x:c>
-      <x:c r="B17" s="46" t="str">
+      <x:c r="B20" s="60" t="str">
         <x:v>literal</x:v>
       </x:c>
-      <x:c r="C17" s="51" t="b">
+      <x:c r="C20" s="70" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D17" s="46" t="str">
+      <x:c r="D20" s="60" t="str">
         <x:v>Fixed backend default</x:v>
       </x:c>
-      <x:c r="E17" s="41" t="str">
+      <x:c r="E20" s="60" t="str">
         <x:v>Request ODB extraction when solver output exists.</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="15" hidden="0" customHeight="1">
-      <x:c r="A18" s="40" t="str">
+    <x:row r="21" ht="15" hidden="0" customHeight="1">
+      <x:c r="A21" s="60" t="str">
         <x:v>solver.step_time</x:v>
       </x:c>
-      <x:c r="B18" s="46" t="str">
+      <x:c r="B21" s="60" t="str">
         <x:v>literal</x:v>
       </x:c>
-      <x:c r="C18" s="46" t="n">
+      <x:c r="C21" s="60" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D18" s="46" t="str">
+      <x:c r="D21" s="60" t="str">
         <x:v>Fixed backend default</x:v>
       </x:c>
-      <x:c r="E18" s="41" t="str">
+      <x:c r="E21" s="60" t="str">
         <x:v>Abaqus step time.</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="15" hidden="0" customHeight="1">
-      <x:c r="A19" s="40" t="str">
+    <x:row r="22" ht="15" hidden="0" customHeight="1">
+      <x:c r="A22" s="60" t="str">
         <x:v>solver.initial_increment</x:v>
       </x:c>
-      <x:c r="B19" s="46" t="str">
+      <x:c r="B22" s="60" t="str">
         <x:v>literal</x:v>
       </x:c>
-      <x:c r="C19" s="46" t="n">
+      <x:c r="C22" s="60" t="n">
         <x:v>0.00001</x:v>
       </x:c>
-      <x:c r="D19" s="46" t="str">
+      <x:c r="D22" s="60" t="str">
         <x:v>Fixed backend default</x:v>
       </x:c>
-      <x:c r="E19" s="41" t="str">
+      <x:c r="E22" s="60" t="str">
         <x:v>Initial increment.</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="15" hidden="0" customHeight="1">
-      <x:c r="A20" s="40" t="str">
+    <x:row r="23" ht="15" hidden="0" customHeight="1">
+      <x:c r="A23" s="60" t="str">
         <x:v>solver.minimum_increment</x:v>
       </x:c>
-      <x:c r="B20" s="46" t="str">
+      <x:c r="B23" s="60" t="str">
         <x:v>literal</x:v>
       </x:c>
-      <x:c r="C20" s="46" t="n">
+      <x:c r="C23" s="60" t="n">
         <x:v>1e-11</x:v>
       </x:c>
-      <x:c r="D20" s="46" t="str">
+      <x:c r="D23" s="60" t="str">
         <x:v>Fixed backend default</x:v>
       </x:c>
-      <x:c r="E20" s="41" t="str">
+      <x:c r="E23" s="60" t="str">
         <x:v>Minimum increment.</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="15" hidden="0" customHeight="1">
-      <x:c r="A21" s="40" t="str">
+    <x:row r="24" ht="15" hidden="0" customHeight="1">
+      <x:c r="A24" s="60" t="str">
         <x:v>solver.maximum_increment</x:v>
       </x:c>
-      <x:c r="B21" s="46" t="str">
+      <x:c r="B24" s="60" t="str">
         <x:v>literal</x:v>
       </x:c>
-      <x:c r="C21" s="46" t="n">
+      <x:c r="C24" s="60" t="n">
         <x:v>0.001</x:v>
       </x:c>
-      <x:c r="D21" s="46" t="str">
+      <x:c r="D24" s="60" t="str">
         <x:v>Fixed backend default</x:v>
       </x:c>
-      <x:c r="E21" s="41" t="str">
+      <x:c r="E24" s="60" t="str">
         <x:v>Maximum increment.</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="15" hidden="0" customHeight="1">
-      <x:c r="A22" s="40" t="str">
+    <x:row r="25" ht="15" hidden="0" customHeight="1">
+      <x:c r="A25" s="60" t="str">
         <x:v>solver.max_num_increments</x:v>
       </x:c>
-      <x:c r="B22" s="46" t="str">
+      <x:c r="B25" s="60" t="str">
         <x:v>literal</x:v>
       </x:c>
-      <x:c r="C22" s="46" t="n">
+      <x:c r="C25" s="60" t="n">
         <x:v>10000</x:v>
       </x:c>
-      <x:c r="D22" s="46" t="str">
+      <x:c r="D25" s="60" t="str">
         <x:v>Fixed backend default</x:v>
       </x:c>
-      <x:c r="E22" s="41" t="str">
+      <x:c r="E25" s="60" t="str">
         <x:v>Maximum increments.</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="15" hidden="0" customHeight="1">
-      <x:c r="A23" s="40" t="str">
+    <x:row r="26" ht="15" hidden="0" customHeight="1">
+      <x:c r="A26" s="60" t="str">
         <x:v>solver.nlgeom</x:v>
       </x:c>
-      <x:c r="B23" s="46" t="str">
+      <x:c r="B26" s="60" t="str">
         <x:v>literal</x:v>
       </x:c>
-      <x:c r="C23" s="51" t="b">
+      <x:c r="C26" s="70" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D23" s="46" t="str">
+      <x:c r="D26" s="60" t="str">
         <x:v>Fixed backend default</x:v>
       </x:c>
-      <x:c r="E23" s="41" t="str">
+      <x:c r="E26" s="60" t="str">
         <x:v>Nonlinear geometry flag.</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="15" hidden="0" customHeight="1">
-      <x:c r="A24" s="40" t="str">
+    <x:row r="27" ht="15" hidden="0" customHeight="1">
+      <x:c r="A27" s="60" t="str">
         <x:v>solver.stabilization_enabled</x:v>
       </x:c>
-      <x:c r="B24" s="46" t="str">
+      <x:c r="B27" s="60" t="str">
         <x:v>literal</x:v>
       </x:c>
-      <x:c r="C24" s="51" t="b">
+      <x:c r="C27" s="70" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D24" s="46" t="str">
+      <x:c r="D27" s="60" t="str">
         <x:v>Fixed backend default</x:v>
       </x:c>
-      <x:c r="E24" s="41" t="str">
+      <x:c r="E27" s="60" t="str">
         <x:v>Stabilization request.</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" ht="15" hidden="0" customHeight="1">
-      <x:c r="A25" s="40" t="str">
+    <x:row r="28" ht="15" hidden="0" customHeight="1">
+      <x:c r="A28" s="60" t="str">
         <x:v>solver.stabilization_factor</x:v>
       </x:c>
-      <x:c r="B25" s="46" t="str">
+      <x:c r="B28" s="60" t="str">
         <x:v>literal</x:v>
       </x:c>
-      <x:c r="C25" s="46" t="n">
+      <x:c r="C28" s="60" t="n">
         <x:v>0.0002</x:v>
       </x:c>
-      <x:c r="D25" s="46" t="str">
+      <x:c r="D28" s="60" t="str">
         <x:v>Fixed backend default</x:v>
       </x:c>
-      <x:c r="E25" s="41" t="str">
+      <x:c r="E28" s="60" t="str">
         <x:v>Stabilization factor.</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="15" hidden="0" customHeight="1">
-      <x:c r="A26" s="40" t="str">
+    <x:row r="29" ht="15" hidden="0" customHeight="1">
+      <x:c r="A29" s="60" t="str">
         <x:v>output_requests.history</x:v>
       </x:c>
-      <x:c r="B26" s="46" t="str">
+      <x:c r="B29" s="60" t="str">
         <x:v>literal</x:v>
       </x:c>
-      <x:c r="C26" s="46" t="str">
+      <x:c r="C29" s="60" t="str">
         <x:v>UR2, RM2</x:v>
       </x:c>
-      <x:c r="D26" s="46" t="str">
+      <x:c r="D29" s="60" t="str">
         <x:v>Fixed backend default</x:v>
       </x:c>
-      <x:c r="E26" s="41" t="str">
+      <x:c r="E29" s="60" t="str">
         <x:v>History outputs for rotation/reaction moment.</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="15" hidden="0" customHeight="1">
-      <x:c r="A27" s="40" t="str">
+    <x:row r="30" ht="15" hidden="0" customHeight="1">
+      <x:c r="A30" s="60" t="str">
         <x:v>output_requests.field</x:v>
       </x:c>
-      <x:c r="B27" s="46" t="str">
+      <x:c r="B30" s="60" t="str">
         <x:v>literal</x:v>
       </x:c>
-      <x:c r="C27" s="46" t="str">
+      <x:c r="C30" s="60" t="str">
         <x:v>U_UR, RF_RM, S, CPRESS, COPEN, CSLIP, CSHEAR</x:v>
       </x:c>
-      <x:c r="D27" s="46" t="str">
+      <x:c r="D30" s="60" t="str">
         <x:v>Fixed backend default</x:v>
       </x:c>
-      <x:c r="E27" s="41" t="str">
+      <x:c r="E30" s="60" t="str">
         <x:v>Field outputs for local contact/stress review.</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" ht="15" hidden="0" customHeight="1">
-      <x:c r="A28" s="40" t="str">
+    <x:row r="31" ht="15" hidden="0" customHeight="1">
+      <x:c r="A31" s="60" t="str">
         <x:v>modeling.model_type</x:v>
       </x:c>
-      <x:c r="B28" s="46" t="str">
+      <x:c r="B31" s="60" t="str">
         <x:v>literal</x:v>
       </x:c>
-      <x:c r="C28" s="46" t="str">
+      <x:c r="C31" s="60" t="str">
         <x:v>full_3d</x:v>
       </x:c>
-      <x:c r="D28" s="46" t="str">
+      <x:c r="D31" s="60" t="str">
         <x:v>Fixed backend default</x:v>
       </x:c>
-      <x:c r="E28" s="41" t="str">
+      <x:c r="E31" s="60" t="str">
         <x:v>Current implemented path.</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="15" hidden="0" customHeight="1">
-      <x:c r="A29" s="40" t="str">
+    <x:row r="32" ht="15" hidden="0" customHeight="1">
+      <x:c r="A32" s="68" t="str">
         <x:v>modeling.equivalent_model_level</x:v>
       </x:c>
-      <x:c r="B29" s="46" t="str">
+      <x:c r="B32" s="68" t="str">
         <x:v>literal</x:v>
       </x:c>
-      <x:c r="C29" s="46" t="n">
+      <x:c r="C32" s="68" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D29" s="46" t="str">
+      <x:c r="D32" s="68" t="str">
         <x:v>Fixed backend default</x:v>
       </x:c>
-      <x:c r="E29" s="41" t="str">
+      <x:c r="E32" s="68" t="str">
         <x:v>Equivalent model support remains future/stretch.</x:v>
       </x:c>
     </x:row>
-    <x:row r="30" ht="15" hidden="0" customHeight="1">
-      <x:c r="A30" s="40" t="str">
+    <x:row r="33" ht="15" hidden="0" customHeight="1">
+      <x:c r="A33" s="68" t="str">
         <x:v>backend_output_contract.required_csv</x:v>
       </x:c>
-      <x:c r="B30" s="46" t="str">
+      <x:c r="B33" s="68" t="str">
         <x:v>literal</x:v>
       </x:c>
-      <x:c r="C30" s="46" t="str">
+      <x:c r="C33" s="68" t="str">
         <x:v>result_data.csv</x:v>
       </x:c>
-      <x:c r="D30" s="46" t="str">
+      <x:c r="D33" s="68" t="str">
         <x:v>Fixed backend contract</x:v>
       </x:c>
-      <x:c r="E30" s="41" t="str">
+      <x:c r="E33" s="68" t="str">
         <x:v>Primary result CSV name.</x:v>
       </x:c>
     </x:row>
-    <x:row r="31" ht="15" hidden="0" customHeight="1">
-      <x:c r="A31" s="42" t="str">
+    <x:row r="34" ht="15" hidden="0" customHeight="1">
+      <x:c r="A34" s="68" t="str">
         <x:v>backend_output_contract.required_columns</x:v>
       </x:c>
-      <x:c r="B31" s="47" t="str">
+      <x:c r="B34" s="68" t="str">
         <x:v>literal</x:v>
       </x:c>
-      <x:c r="C31" s="47" t="str">
+      <x:c r="C34" s="68" t="str">
         <x:v>curvature_1_per_m, moment_kn_m</x:v>
       </x:c>
-      <x:c r="D31" s="47" t="str">
+      <x:c r="D34" s="68" t="str">
         <x:v>Fixed backend contract</x:v>
       </x:c>
-      <x:c r="E31" s="43" t="str">
+      <x:c r="E34" s="68" t="str">
         <x:v>Required result columns.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="15" hidden="0" customHeight="1">
+      <x:c r="A35" s="68" t="str">
+        <x:v>backend_output_contract.optional_odb</x:v>
+      </x:c>
+      <x:c r="B35" s="68" t="str">
+        <x:v>literal</x:v>
+      </x:c>
+      <x:c r="C35" s="68" t="str">
+        <x:v>*.odb</x:v>
+      </x:c>
+      <x:c r="D35" s="68" t="str">
+        <x:v>Fixed backend contract</x:v>
+      </x:c>
+      <x:c r="E35" s="68" t="str">
+        <x:v>ODB is optional but expected for research-quality extraction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="15" hidden="0" customHeight="1">
+      <x:c r="A36" s="68" t="str">
+        <x:v>backend_exchange_contract.input_source_of_truth</x:v>
+      </x:c>
+      <x:c r="B36" s="68" t="str">
+        <x:v>literal</x:v>
+      </x:c>
+      <x:c r="C36" s="68" t="str">
+        <x:v>input_data.json</x:v>
+      </x:c>
+      <x:c r="D36" s="68" t="str">
+        <x:v>Fixed exchange contract</x:v>
+      </x:c>
+      <x:c r="E36" s="68" t="str">
+        <x:v>GUI/backend source of truth for one job folder.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="15" hidden="0" customHeight="1">
+      <x:c r="A37" s="68" t="str">
+        <x:v>backend_exchange_contract.job_folder_files_written_by_gui</x:v>
+      </x:c>
+      <x:c r="B37" s="68" t="str">
+        <x:v>literal</x:v>
+      </x:c>
+      <x:c r="C37" s="68" t="str">
+        <x:v>input_data.json, units_manifest.json, BACKEND_CONTRACT.md, abaqus_runner.py, sclas_odb_extractor.py</x:v>
+      </x:c>
+      <x:c r="D37" s="68" t="str">
+        <x:v>Fixed exchange contract</x:v>
+      </x:c>
+      <x:c r="E37" s="68" t="str">
+        <x:v>Files copied/written before backend execution.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="15" hidden="0" customHeight="1">
+      <x:c r="A38" s="68" t="str">
+        <x:v>backend_exchange_contract.gui_reads_after_backend</x:v>
+      </x:c>
+      <x:c r="B38" s="68" t="str">
+        <x:v>literal</x:v>
+      </x:c>
+      <x:c r="C38" s="68" t="str">
+        <x:v>result_data.csv, result_summary.json, abaqus_mesh_manifest.json, odb_extraction_summary.json</x:v>
+      </x:c>
+      <x:c r="D38" s="68" t="str">
+        <x:v>Fixed exchange contract</x:v>
+      </x:c>
+      <x:c r="E38" s="68" t="str">
+        <x:v>Files the GUI can read after backend execution.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>